<commit_message>
chore(data): batch update intraday vendas - 10:00:02
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,6 +482,82 @@
         <is>
           <t>TOTAL_VALOR_VENDA</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>145</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>139865</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2500455</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>46419</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H2" t="n">
+        <v>794365</v>
+      </c>
+      <c r="I2" t="n">
+        <v>12.68</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>125</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>142672</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>25E02W</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H3" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I3" t="n">
+        <v>39.28</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 10:15:03
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -516,10 +516,10 @@
         <v>794365</v>
       </c>
       <c r="I2" t="n">
-        <v>12.68</v>
+        <v>12.71</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>12.71</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 10:45:06
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -554,10 +554,10 @@
         <v>789429</v>
       </c>
       <c r="I3" t="n">
-        <v>39.28</v>
+        <v>39.31</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:15:03
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,35 +491,35 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>139865</v>
+        <v>103195</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>4R7537</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H2" t="n">
-        <v>794365</v>
+        <v>53333</v>
       </c>
       <c r="I2" t="n">
-        <v>25.42</v>
+        <v>204.23</v>
       </c>
       <c r="J2" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -529,35 +529,35 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>142672</v>
+        <v>139865</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H3" t="n">
-        <v>789429</v>
+        <v>794365</v>
       </c>
       <c r="I3" t="n">
-        <v>39.31</v>
+        <v>25.42</v>
       </c>
       <c r="J3" t="n">
-        <v>39.31</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="4">
@@ -575,11 +575,11 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>92720</v>
+        <v>142672</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
@@ -589,13 +589,13 @@
         <v>46259</v>
       </c>
       <c r="H4" t="n">
-        <v>37273</v>
+        <v>789429</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
       <c r="J4" t="n">
-        <v>6.88</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="5">
@@ -605,35 +605,149 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>88358</v>
+        <v>142886</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H5" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I5" t="n">
+        <v>32.62</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>125</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>92720</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>4V3334</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H6" t="n">
+        <v>37273</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>6.88</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>125</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>88358</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>GRA01137</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H7" t="n">
         <v>793056</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I7" t="n">
         <v>0</v>
       </c>
-      <c r="J5" t="n">
+      <c r="J7" t="n">
         <v>21.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>125</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H8" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I8" t="n">
+        <v>51.33</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 11:30:04
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,27 +499,27 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>103195</v>
+        <v>73911</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4R7537</t>
+          <t>576357</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H2" t="n">
-        <v>53333</v>
+        <v>47252</v>
       </c>
       <c r="I2" t="n">
-        <v>204.23</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>65.81</v>
       </c>
     </row>
     <row r="3">
@@ -529,35 +529,35 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>139865</v>
+        <v>103195</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>4R7537</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H3" t="n">
-        <v>794365</v>
+        <v>53333</v>
       </c>
       <c r="I3" t="n">
-        <v>25.42</v>
+        <v>204.3</v>
       </c>
       <c r="J3" t="n">
-        <v>25.42</v>
+        <v>204.3</v>
       </c>
     </row>
     <row r="4">
@@ -567,35 +567,35 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>142672</v>
+        <v>139865</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H4" t="n">
-        <v>789429</v>
+        <v>794365</v>
       </c>
       <c r="I4" t="n">
-        <v>39.31</v>
+        <v>25.42</v>
       </c>
       <c r="J4" t="n">
-        <v>39.31</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="5">
@@ -605,35 +605,35 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>142886</v>
+        <v>142672</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H5" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I5" t="n">
-        <v>32.62</v>
+        <v>39.31</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="6">
@@ -643,35 +643,35 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>92720</v>
+        <v>142886</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H6" t="n">
-        <v>37273</v>
+        <v>789423</v>
       </c>
       <c r="I6" t="n">
+        <v>32.62</v>
+      </c>
+      <c r="J6" t="n">
         <v>0</v>
-      </c>
-      <c r="J6" t="n">
-        <v>6.88</v>
       </c>
     </row>
     <row r="7">
@@ -689,11 +689,11 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>88358</v>
+        <v>92720</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -703,13 +703,13 @@
         <v>46259</v>
       </c>
       <c r="H7" t="n">
-        <v>793056</v>
+        <v>37273</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>21.4</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="8">
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>106364</v>
+        <v>88358</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -741,13 +741,51 @@
         <v>46259</v>
       </c>
       <c r="H8" t="n">
+        <v>793056</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>125</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H9" t="n">
         <v>65455</v>
       </c>
-      <c r="I8" t="n">
-        <v>51.33</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
+      <c r="I9" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="J9" t="n">
+        <v>51.35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 12:00:03
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -563,39 +563,39 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>139865</v>
+        <v>79375</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>B25H1773</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H4" t="n">
-        <v>794365</v>
+        <v>47252</v>
       </c>
       <c r="I4" t="n">
-        <v>25.42</v>
+        <v>150.28</v>
       </c>
       <c r="J4" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -605,35 +605,35 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>142672</v>
+        <v>139865</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H5" t="n">
-        <v>789429</v>
+        <v>794365</v>
       </c>
       <c r="I5" t="n">
-        <v>39.31</v>
+        <v>25.42</v>
       </c>
       <c r="J5" t="n">
-        <v>39.31</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="6">
@@ -643,35 +643,35 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>142886</v>
+        <v>142672</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H6" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I6" t="n">
-        <v>32.62</v>
+        <v>39.31</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="7">
@@ -681,35 +681,35 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>92720</v>
+        <v>142886</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H7" t="n">
-        <v>37273</v>
+        <v>789423</v>
       </c>
       <c r="I7" t="n">
+        <v>32.62</v>
+      </c>
+      <c r="J7" t="n">
         <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>6.88</v>
       </c>
     </row>
     <row r="8">
@@ -727,11 +727,11 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>88358</v>
+        <v>92720</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -741,13 +741,13 @@
         <v>46259</v>
       </c>
       <c r="H8" t="n">
-        <v>793056</v>
+        <v>37273</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>21.4</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="9">
@@ -765,11 +765,11 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>106364</v>
+        <v>88358</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
@@ -779,12 +779,50 @@
         <v>46259</v>
       </c>
       <c r="H9" t="n">
+        <v>793056</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>125</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H10" t="n">
         <v>65455</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I10" t="n">
         <v>51.35</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J10" t="n">
         <v>51.35</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:16:38
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -525,188 +525,188 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>103195</v>
+        <v>83810</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>4R7537</t>
+          <t>0030382</t>
         </is>
       </c>
       <c r="F3" s="2" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H3" t="n">
-        <v>53333</v>
+        <v>33057</v>
       </c>
       <c r="I3" t="n">
-        <v>204.3</v>
+        <v>18.7</v>
       </c>
       <c r="J3" t="n">
-        <v>204.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>79375</v>
+        <v>103195</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>B25H1773</t>
+          <t>4R7537</t>
         </is>
       </c>
       <c r="F4" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H4" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I4" t="n">
-        <v>150.28</v>
+        <v>204.3</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>204.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>139865</v>
+        <v>993207</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>A36E00325</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H5" t="n">
-        <v>794365</v>
+        <v>790283</v>
       </c>
       <c r="I5" t="n">
-        <v>25.42</v>
+        <v>6.25</v>
       </c>
       <c r="J5" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>142672</v>
+        <v>173</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>3QM99</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46508</v>
+        <v>46327</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H6" t="n">
-        <v>789429</v>
+        <v>33766</v>
       </c>
       <c r="I6" t="n">
-        <v>39.31</v>
+        <v>20.64</v>
       </c>
       <c r="J6" t="n">
-        <v>39.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>142886</v>
+        <v>79375</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>B25H1773</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>46388</v>
+        <v>46478</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H7" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I7" t="n">
-        <v>32.62</v>
+        <v>150.28</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -719,35 +719,35 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>92720</v>
+        <v>139865</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H8" t="n">
-        <v>37273</v>
+        <v>794365</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="J8" t="n">
-        <v>6.88</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="9">
@@ -765,65 +765,597 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>88358</v>
+        <v>98663</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H9" t="n">
-        <v>793056</v>
+        <v>37273</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>21.4</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>39</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>153462</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>68340022</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H10" t="n">
+        <v>30791</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1302.28</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B11" t="n">
+        <v>145</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>158962</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>41103077</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H11" t="n">
+        <v>793718</v>
+      </c>
+      <c r="I11" t="n">
+        <v>196.61</v>
+      </c>
+      <c r="J11" t="n">
+        <v>196.61</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>147</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>120901</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0029956</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>46327</v>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H12" t="n">
+        <v>33057</v>
+      </c>
+      <c r="I12" t="n">
+        <v>81.26000000000001</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>147</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>155008</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>255239</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H13" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I13" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>147</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>110370</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>B25A1125</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H14" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I14" t="n">
+        <v>62.45</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>147</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>147194</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>B24G9303</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H15" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I15" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>147</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>81973</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>B25A0083</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>46419</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H16" t="n">
+        <v>47252</v>
+      </c>
+      <c r="I16" t="n">
+        <v>6.23</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>125</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D17" t="n">
+        <v>142672</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>25E02W</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H17" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I17" t="n">
+        <v>39.31</v>
+      </c>
+      <c r="J17" t="n">
+        <v>39.31</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>111</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>142886</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0000269338</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G18" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H18" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I18" t="n">
+        <v>32.62</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>125</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>159083</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2504659</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G19" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H19" t="n">
+        <v>794365</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>88.59999999999999</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>125</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>92720</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>4V3334</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H20" t="n">
+        <v>37273</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>6.88</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>111</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>140760</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0000273697</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H21" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I21" t="n">
+        <v>37.39</v>
+      </c>
+      <c r="J21" t="n">
+        <v>37.39</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>125</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>88358</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>GRA01137</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G22" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H22" t="n">
+        <v>793056</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>125</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
         <v>106364</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>BR183284</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F23" s="2" t="n">
         <v>46508</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H10" t="n">
+      <c r="G23" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H23" t="n">
         <v>65455</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I23" t="n">
         <v>51.35</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J23" t="n">
         <v>51.35</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>147</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H24" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I24" t="n">
+        <v>10.42</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 13:30:02
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,10 +554,10 @@
         <v>33057</v>
       </c>
       <c r="I3" t="n">
-        <v>18.7</v>
+        <v>18.72</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="4">
@@ -601,39 +601,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>993207</v>
+        <v>159130</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>A36E00325</t>
+          <t>25D22K</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H5" t="n">
-        <v>790283</v>
+        <v>789429</v>
       </c>
       <c r="I5" t="n">
-        <v>6.25</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1567.66</v>
       </c>
     </row>
     <row r="6">
@@ -651,27 +651,27 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>173</v>
+        <v>993207</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3QM99</t>
+          <t>A36E00325</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46327</v>
+        <v>46388</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H6" t="n">
-        <v>33766</v>
+        <v>790283</v>
       </c>
       <c r="I6" t="n">
-        <v>20.64</v>
+        <v>6.25</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="7">
@@ -689,65 +689,65 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>79375</v>
+        <v>173</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>B25H1773</t>
+          <t>3QM99</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>46478</v>
+        <v>46327</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H7" t="n">
-        <v>47252</v>
+        <v>33766</v>
       </c>
       <c r="I7" t="n">
-        <v>150.28</v>
+        <v>20.66</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>20.66</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>139865</v>
+        <v>79375</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>B25H1773</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H8" t="n">
-        <v>794365</v>
+        <v>47252</v>
       </c>
       <c r="I8" t="n">
-        <v>25.42</v>
+        <v>150.28</v>
       </c>
       <c r="J8" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -757,35 +757,35 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>98663</v>
+        <v>139865</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4R6305</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H9" t="n">
-        <v>37273</v>
+        <v>794365</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="J9" t="n">
-        <v>29.51</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="10">
@@ -803,27 +803,27 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>153462</v>
+        <v>142466</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>25I07B</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
-        <v>46478</v>
+        <v>46419</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H10" t="n">
-        <v>30791</v>
+        <v>789429</v>
       </c>
       <c r="I10" t="n">
-        <v>1302.28</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>417.34</v>
       </c>
     </row>
     <row r="11">
@@ -833,108 +833,108 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>158962</v>
+        <v>98663</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H11" t="n">
-        <v>793718</v>
+        <v>37273</v>
       </c>
       <c r="I11" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>196.61</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>147</v>
+        <v>80</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>120901</v>
+        <v>118036</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>46327</v>
+        <v>46508</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H12" t="n">
-        <v>33057</v>
+        <v>790808</v>
       </c>
       <c r="I12" t="n">
-        <v>81.26000000000001</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>155008</v>
+        <v>153462</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46388</v>
+        <v>46478</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H13" t="n">
-        <v>790283</v>
+        <v>30791</v>
       </c>
       <c r="I13" t="n">
-        <v>18.7</v>
+        <v>1302.28</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
@@ -943,39 +943,39 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>110370</v>
+        <v>158962</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H14" t="n">
-        <v>47252</v>
+        <v>793718</v>
       </c>
       <c r="I14" t="n">
-        <v>62.45</v>
+        <v>196.61</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="15">
@@ -993,24 +993,24 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>147194</v>
+        <v>120901</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46388</v>
+        <v>46327</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H15" t="n">
-        <v>33928</v>
+        <v>33057</v>
       </c>
       <c r="I15" t="n">
-        <v>7.99</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -1031,87 +1031,87 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>81973</v>
+        <v>155008</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H16" t="n">
-        <v>47252</v>
+        <v>790283</v>
       </c>
       <c r="I16" t="n">
-        <v>6.23</v>
+        <v>18.72</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>142672</v>
+        <v>110370</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I17" t="n">
-        <v>39.31</v>
+        <v>62.52</v>
       </c>
       <c r="J17" t="n">
-        <v>39.31</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>142886</v>
+        <v>147194</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -1121,10 +1121,10 @@
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I18" t="n">
-        <v>32.62</v>
+        <v>7.99</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1133,77 +1133,77 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>159083</v>
+        <v>148828</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>794365</v>
+        <v>792019</v>
       </c>
       <c r="I19" t="n">
+        <v>93.70999999999999</v>
+      </c>
+      <c r="J19" t="n">
         <v>0</v>
-      </c>
-      <c r="J19" t="n">
-        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>92720</v>
+        <v>81973</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>37273</v>
+        <v>47252</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>6.24</v>
       </c>
       <c r="J20" t="n">
-        <v>6.88</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="21">
@@ -1213,35 +1213,35 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>140760</v>
+        <v>142672</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I21" t="n">
-        <v>37.39</v>
+        <v>39.31</v>
       </c>
       <c r="J21" t="n">
-        <v>37.39</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="22">
@@ -1251,35 +1251,35 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>88358</v>
+        <v>142886</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>793056</v>
+        <v>789423</v>
       </c>
       <c r="I22" t="n">
+        <v>32.62</v>
+      </c>
+      <c r="J22" t="n">
         <v>0</v>
-      </c>
-      <c r="J22" t="n">
-        <v>21.4</v>
       </c>
     </row>
     <row r="23">
@@ -1297,65 +1297,255 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>106364</v>
+        <v>159083</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>65455</v>
+        <v>794365</v>
       </c>
       <c r="I23" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>51.35</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>125</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>92720</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>4V3334</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G24" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H24" t="n">
+        <v>37273</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>6.88</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>111</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>140760</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0000273697</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G25" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H25" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I25" t="n">
+        <v>37.39</v>
+      </c>
+      <c r="J25" t="n">
+        <v>37.39</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B26" t="n">
         <v>147</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="D26" t="n">
+        <v>84824</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>FKP06475</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H26" t="n">
+        <v>789662</v>
+      </c>
+      <c r="I26" t="n">
+        <v>27.31</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>125</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>88358</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>GRA01137</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G27" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H27" t="n">
+        <v>793056</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>21.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>125</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H28" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I28" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="J28" t="n">
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>147</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
         <v>148816</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>T16725</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F29" s="2" t="n">
         <v>46478</v>
       </c>
-      <c r="G24" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H24" t="n">
+      <c r="G29" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H29" t="n">
         <v>33928</v>
       </c>
-      <c r="I24" t="n">
-        <v>10.42</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0</v>
+      <c r="I29" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J29" t="n">
+        <v>10.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:15:03
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -630,7 +630,7 @@
         <v>789429</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>62.71</v>
       </c>
       <c r="J5" t="n">
         <v>1567.66</v>
@@ -1124,10 +1124,10 @@
         <v>5582</v>
       </c>
       <c r="I18" t="n">
-        <v>80.5</v>
+        <v>80.55</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="19">
@@ -1162,10 +1162,10 @@
         <v>794919</v>
       </c>
       <c r="I19" t="n">
-        <v>150.94</v>
+        <v>150.95</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="20">
@@ -1238,10 +1238,10 @@
         <v>789423</v>
       </c>
       <c r="I21" t="n">
-        <v>510.36</v>
+        <v>510.49</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="22">
@@ -1314,10 +1314,10 @@
         <v>31305</v>
       </c>
       <c r="I23" t="n">
-        <v>184.96</v>
+        <v>185.14</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="24">
@@ -1428,10 +1428,10 @@
         <v>789423</v>
       </c>
       <c r="I26" t="n">
-        <v>283.55</v>
+        <v>283.62</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="27">
@@ -1580,10 +1580,10 @@
         <v>789423</v>
       </c>
       <c r="I30" t="n">
-        <v>158.74</v>
+        <v>158.77</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="31">
@@ -1817,38 +1817,76 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>39</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G37" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H37" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>12.53</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B38" t="n">
         <v>147</v>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D38" t="n">
         <v>148816</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>T16725</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F38" s="2" t="n">
         <v>46478</v>
       </c>
-      <c r="G37" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H37" t="n">
+      <c r="G38" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H38" t="n">
         <v>33928</v>
       </c>
-      <c r="I37" t="n">
+      <c r="I38" t="n">
         <v>10.43</v>
       </c>
-      <c r="J37" t="n">
+      <c r="J38" t="n">
         <v>10.43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 14:30:04
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -601,77 +601,77 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>159130</v>
+        <v>123463</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>25D22K</t>
+          <t>A07A00125</t>
         </is>
       </c>
       <c r="F5" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H5" t="n">
-        <v>789429</v>
+        <v>31305</v>
       </c>
       <c r="I5" t="n">
-        <v>62.71</v>
+        <v>26.23</v>
       </c>
       <c r="J5" t="n">
-        <v>1567.66</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>993207</v>
+        <v>159130</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>A36E00325</t>
+          <t>25D22K</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H6" t="n">
-        <v>790283</v>
+        <v>789429</v>
       </c>
       <c r="I6" t="n">
-        <v>6.25</v>
+        <v>62.71</v>
       </c>
       <c r="J6" t="n">
-        <v>6.25</v>
+        <v>1567.66</v>
       </c>
     </row>
     <row r="7">
@@ -689,27 +689,27 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>173</v>
+        <v>993207</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3QM99</t>
+          <t>A36E00325</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
-        <v>46327</v>
+        <v>46388</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H7" t="n">
-        <v>33766</v>
+        <v>790283</v>
       </c>
       <c r="I7" t="n">
-        <v>20.66</v>
+        <v>6.25</v>
       </c>
       <c r="J7" t="n">
-        <v>20.66</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="8">
@@ -727,87 +727,87 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>79375</v>
+        <v>173</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>B25H1773</t>
+          <t>3QM99</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
-        <v>46478</v>
+        <v>46327</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H8" t="n">
-        <v>47252</v>
+        <v>33766</v>
       </c>
       <c r="I8" t="n">
-        <v>150.28</v>
+        <v>20.66</v>
       </c>
       <c r="J8" t="n">
-        <v>0</v>
+        <v>20.66</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>139865</v>
+        <v>79375</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>B25H1773</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H9" t="n">
-        <v>794365</v>
+        <v>47252</v>
       </c>
       <c r="I9" t="n">
-        <v>25.42</v>
+        <v>150.28</v>
       </c>
       <c r="J9" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>142466</v>
+        <v>139865</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>25I07B</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
@@ -817,51 +817,51 @@
         <v>46259</v>
       </c>
       <c r="H10" t="n">
-        <v>789429</v>
+        <v>794365</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
       <c r="J10" t="n">
-        <v>417.34</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>155114</v>
+        <v>142466</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0000267854</t>
+          <t>25I07B</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>46327</v>
+        <v>46419</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H11" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I11" t="n">
-        <v>84.31</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>417.34</v>
       </c>
     </row>
     <row r="12">
@@ -871,35 +871,35 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>98663</v>
+        <v>155114</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4R6305</t>
+          <t>0000267854</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>46447</v>
+        <v>46327</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H12" t="n">
-        <v>37273</v>
+        <v>789423</v>
       </c>
       <c r="I12" t="n">
+        <v>84.31</v>
+      </c>
+      <c r="J12" t="n">
         <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>29.51</v>
       </c>
     </row>
     <row r="13">
@@ -909,73 +909,73 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>115223</v>
+        <v>98663</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H13" t="n">
-        <v>789423</v>
+        <v>37273</v>
       </c>
       <c r="I13" t="n">
-        <v>62.07</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H14" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I14" t="n">
+        <v>62.07</v>
+      </c>
+      <c r="J14" t="n">
         <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>346.2</v>
       </c>
     </row>
     <row r="15">
@@ -985,149 +985,149 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>153462</v>
+        <v>118036</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H15" t="n">
-        <v>30791</v>
+        <v>790808</v>
       </c>
       <c r="I15" t="n">
-        <v>1302.28</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>158962</v>
+        <v>153462</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H16" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="I16" t="n">
-        <v>196.61</v>
+        <v>1302.28</v>
       </c>
       <c r="J16" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>120901</v>
+        <v>158962</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46327</v>
+        <v>46508</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>33057</v>
+        <v>793718</v>
       </c>
       <c r="I17" t="n">
-        <v>81.26000000000001</v>
+        <v>196.61</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>152839</v>
+        <v>120901</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46388</v>
+        <v>46327</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>5582</v>
+        <v>33057</v>
       </c>
       <c r="I18" t="n">
-        <v>80.55</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J18" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1145,163 +1145,163 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>154122</v>
+        <v>152839</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>794919</v>
+        <v>5582</v>
       </c>
       <c r="I19" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
       <c r="J19" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>155008</v>
+        <v>154122</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>790283</v>
+        <v>794919</v>
       </c>
       <c r="I20" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
       <c r="J20" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>155969</v>
+        <v>155008</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>789423</v>
+        <v>790283</v>
       </c>
       <c r="I21" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
       <c r="J21" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>110370</v>
+        <v>155969</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I22" t="n">
-        <v>62.52</v>
+        <v>510.49</v>
       </c>
       <c r="J22" t="n">
-        <v>62.52</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>142124</v>
+        <v>110370</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1311,35 +1311,35 @@
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I23" t="n">
-        <v>185.14</v>
+        <v>62.52</v>
       </c>
       <c r="J23" t="n">
-        <v>185.13</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>147194</v>
+        <v>142124</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1349,13 +1349,13 @@
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I24" t="n">
-        <v>7.99</v>
+        <v>185.14</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="25">
@@ -1373,24 +1373,24 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>148828</v>
+        <v>147194</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>792019</v>
+        <v>33928</v>
       </c>
       <c r="I25" t="n">
-        <v>93.70999999999999</v>
+        <v>7.99</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1399,23 +1399,23 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>155970</v>
+        <v>148828</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1425,89 +1425,89 @@
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>789423</v>
+        <v>792019</v>
       </c>
       <c r="I26" t="n">
-        <v>283.62</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>81973</v>
+        <v>155970</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I27" t="n">
-        <v>6.24</v>
+        <v>283.62</v>
       </c>
       <c r="J27" t="n">
-        <v>6.24</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>142672</v>
+        <v>81973</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I28" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
       <c r="J28" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="29">
@@ -1517,57 +1517,57 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>142886</v>
+        <v>142672</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I29" t="n">
-        <v>65.23999999999999</v>
+        <v>39.31</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>155919</v>
+        <v>142886</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -1580,48 +1580,48 @@
         <v>789423</v>
       </c>
       <c r="I30" t="n">
-        <v>158.77</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J30" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>159083</v>
+        <v>155919</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
       <c r="J31" t="n">
-        <v>88.59999999999999</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="32">
@@ -1639,27 +1639,27 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>92720</v>
+        <v>159083</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>37273</v>
+        <v>794365</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>6.88</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="33">
@@ -1669,95 +1669,95 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>140760</v>
+        <v>92720</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>789423</v>
+        <v>37273</v>
       </c>
       <c r="I33" t="n">
-        <v>37.39</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>37.39</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>84824</v>
+        <v>140760</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>789662</v>
+        <v>789423</v>
       </c>
       <c r="I34" t="n">
-        <v>27.31</v>
+        <v>37.39</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>88358</v>
+        <v>84824</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -1767,13 +1767,13 @@
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>793056</v>
+        <v>789662</v>
       </c>
       <c r="I35" t="n">
+        <v>27.31</v>
+      </c>
+      <c r="J35" t="n">
         <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>21.4</v>
       </c>
     </row>
     <row r="36">
@@ -1791,11 +1791,11 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>106364</v>
+        <v>88358</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -1805,35 +1805,35 @@
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>65455</v>
+        <v>793056</v>
       </c>
       <c r="I36" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>51.35</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>146095</v>
+        <v>106364</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -1843,50 +1843,88 @@
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>790283</v>
+        <v>65455</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>51.35</v>
       </c>
       <c r="J37" t="n">
-        <v>12.53</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>39</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G38" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H38" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>12.53</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B39" t="n">
         <v>147</v>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>148816</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>T16725</t>
         </is>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="F39" s="2" t="n">
         <v>46478</v>
       </c>
-      <c r="G38" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H38" t="n">
+      <c r="G39" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H39" t="n">
         <v>33928</v>
       </c>
-      <c r="I38" t="n">
+      <c r="I39" t="n">
         <v>10.43</v>
       </c>
-      <c r="J38" t="n">
+      <c r="J39" t="n">
         <v>10.43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:00:05
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J42"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -706,7 +706,7 @@
         <v>789423</v>
       </c>
       <c r="I7" t="n">
-        <v>44.14</v>
+        <v>80</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -1665,27 +1665,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>155919</v>
+        <v>153194</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
@@ -1694,48 +1694,48 @@
         <v>789423</v>
       </c>
       <c r="I33" t="n">
-        <v>158.77</v>
+        <v>155.28</v>
       </c>
       <c r="J33" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>159083</v>
+        <v>155919</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
       <c r="J34" t="n">
-        <v>88.59999999999999</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="35">
@@ -1753,87 +1753,87 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>92720</v>
+        <v>159083</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>37273</v>
+        <v>794365</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>6.88</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>140760</v>
+        <v>66958</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>789423</v>
+        <v>789525</v>
       </c>
       <c r="I36" t="n">
-        <v>37.39</v>
+        <v>59.32</v>
       </c>
       <c r="J36" t="n">
-        <v>37.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>84824</v>
+        <v>92720</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
@@ -1843,13 +1843,13 @@
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>789662</v>
+        <v>37273</v>
       </c>
       <c r="I37" t="n">
-        <v>27.31</v>
+        <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="38">
@@ -1859,70 +1859,70 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>88358</v>
+        <v>140760</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>793056</v>
+        <v>789423</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
       <c r="J38" t="n">
-        <v>21.4</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>53</v>
+        <v>147</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>105546</v>
+        <v>84824</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>789423</v>
+        <v>789662</v>
       </c>
       <c r="I39" t="n">
-        <v>48.42</v>
+        <v>27.31</v>
       </c>
       <c r="J39" t="n">
         <v>0</v>
@@ -1943,11 +1943,11 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>106364</v>
+        <v>88358</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
@@ -1957,88 +1957,202 @@
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>65455</v>
+        <v>793056</v>
       </c>
       <c r="I40" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>51.35</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>146095</v>
+        <v>105546</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>790283</v>
+        <v>789423</v>
       </c>
       <c r="I41" t="n">
+        <v>186.49</v>
+      </c>
+      <c r="J41" t="n">
         <v>0</v>
-      </c>
-      <c r="J41" t="n">
-        <v>12.53</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>125</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G42" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H42" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I42" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="J42" t="n">
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>96</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>SILAS SALVIANO PRATI</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>142645</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>25E17F</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G43" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H43" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I43" t="n">
+        <v>81.58</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>39</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G44" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H44" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I44" t="n">
+        <v>8.140000000000001</v>
+      </c>
+      <c r="J44" t="n">
+        <v>12.53</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B45" t="n">
         <v>147</v>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D45" t="n">
         <v>148816</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>T16725</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F45" s="2" t="n">
         <v>46478</v>
       </c>
-      <c r="G42" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H42" t="n">
+      <c r="G45" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H45" t="n">
         <v>33928</v>
       </c>
-      <c r="I42" t="n">
+      <c r="I45" t="n">
         <v>10.43</v>
       </c>
-      <c r="J42" t="n">
+      <c r="J45" t="n">
         <v>10.43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:15:05
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,10 +744,10 @@
         <v>789429</v>
       </c>
       <c r="I8" t="n">
-        <v>62.71</v>
+        <v>62.75</v>
       </c>
       <c r="J8" t="n">
-        <v>1567.66</v>
+        <v>1630.4</v>
       </c>
     </row>
     <row r="9">
@@ -934,10 +934,10 @@
         <v>789429</v>
       </c>
       <c r="I13" t="n">
-        <v>39.95</v>
+        <v>39.97</v>
       </c>
       <c r="J13" t="n">
-        <v>417.34</v>
+        <v>457.31</v>
       </c>
     </row>
     <row r="14">
@@ -1171,36 +1171,36 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>120901</v>
+        <v>20206</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46327</v>
+        <v>46508</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>33057</v>
+        <v>789228</v>
       </c>
       <c r="I20" t="n">
-        <v>81.26000000000001</v>
+        <v>33.94</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1209,99 +1209,99 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>152839</v>
+        <v>64130</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46388</v>
+        <v>45870</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>5582</v>
+        <v>30791</v>
       </c>
       <c r="I21" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>80.55</v>
+        <v>118.94</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>154122</v>
+        <v>120901</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46447</v>
+        <v>46327</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>794919</v>
+        <v>33057</v>
       </c>
       <c r="I22" t="n">
-        <v>150.95</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>150.95</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>155008</v>
+        <v>152839</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1311,13 +1311,13 @@
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>790283</v>
+        <v>5582</v>
       </c>
       <c r="I23" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
       <c r="J23" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="24">
@@ -1335,27 +1335,27 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>155969</v>
+        <v>154122</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>789423</v>
+        <v>794919</v>
       </c>
       <c r="I24" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
       <c r="J24" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="25">
@@ -1373,11 +1373,11 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>110370</v>
+        <v>155008</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -1387,13 +1387,13 @@
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>47252</v>
+        <v>790283</v>
       </c>
       <c r="I25" t="n">
-        <v>62.52</v>
+        <v>18.72</v>
       </c>
       <c r="J25" t="n">
-        <v>62.52</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="26">
@@ -1411,27 +1411,27 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>142124</v>
+        <v>155969</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I26" t="n">
-        <v>185.14</v>
+        <v>510.49</v>
       </c>
       <c r="J26" t="n">
-        <v>185.13</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="27">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>147194</v>
+        <v>110370</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -1463,89 +1463,89 @@
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I27" t="n">
-        <v>7.99</v>
+        <v>62.52</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>148828</v>
+        <v>142124</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>792019</v>
+        <v>31305</v>
       </c>
       <c r="I28" t="n">
-        <v>93.70999999999999</v>
+        <v>185.14</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>155970</v>
+        <v>147194</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I29" t="n">
-        <v>283.62</v>
+        <v>7.99</v>
       </c>
       <c r="J29" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -1563,49 +1563,49 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>81973</v>
+        <v>148828</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>47252</v>
+        <v>792019</v>
       </c>
       <c r="I30" t="n">
-        <v>6.24</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J30" t="n">
-        <v>6.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>142672</v>
+        <v>155970</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -1615,73 +1615,73 @@
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>789429</v>
+        <v>789423</v>
       </c>
       <c r="I31" t="n">
-        <v>39.31</v>
+        <v>283.62</v>
       </c>
       <c r="J31" t="n">
-        <v>39.31</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>142886</v>
+        <v>81973</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I32" t="n">
-        <v>65.23999999999999</v>
+        <v>6.24</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>153194</v>
+        <v>142672</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
@@ -1691,35 +1691,35 @@
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I33" t="n">
-        <v>155.28</v>
+        <v>39.31</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>155919</v>
+        <v>142886</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -1732,86 +1732,86 @@
         <v>789423</v>
       </c>
       <c r="I34" t="n">
-        <v>158.77</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J34" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>159083</v>
+        <v>153194</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I35" t="n">
+        <v>155.28</v>
+      </c>
+      <c r="J35" t="n">
         <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>66958</v>
+        <v>155919</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>789525</v>
+        <v>789423</v>
       </c>
       <c r="I36" t="n">
-        <v>59.32</v>
+        <v>158.77</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="37">
@@ -1829,87 +1829,87 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>92720</v>
+        <v>159083</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>37273</v>
+        <v>794365</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>6.88</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>140760</v>
+        <v>66958</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>789423</v>
+        <v>789525</v>
       </c>
       <c r="I38" t="n">
-        <v>37.39</v>
+        <v>59.39</v>
       </c>
       <c r="J38" t="n">
-        <v>37.39</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>84824</v>
+        <v>92720</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
@@ -1919,13 +1919,13 @@
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>789662</v>
+        <v>37273</v>
       </c>
       <c r="I39" t="n">
-        <v>27.31</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="40">
@@ -1935,57 +1935,57 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>88358</v>
+        <v>140760</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>793056</v>
+        <v>789423</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
       <c r="J40" t="n">
-        <v>21.4</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>105546</v>
+        <v>49964</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -1995,10 +1995,10 @@
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>789423</v>
+        <v>789228</v>
       </c>
       <c r="I41" t="n">
-        <v>186.49</v>
+        <v>82.8</v>
       </c>
       <c r="J41" t="n">
         <v>0</v>
@@ -2007,23 +2007,23 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>106364</v>
+        <v>84824</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
@@ -2033,35 +2033,35 @@
         <v>46259</v>
       </c>
       <c r="H42" t="n">
-        <v>65455</v>
+        <v>789662</v>
       </c>
       <c r="I42" t="n">
-        <v>51.35</v>
+        <v>27.31</v>
       </c>
       <c r="J42" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>142645</v>
+        <v>88358</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
@@ -2071,73 +2071,73 @@
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>789429</v>
+        <v>793056</v>
       </c>
       <c r="I43" t="n">
-        <v>81.58</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>146095</v>
+        <v>105546</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H44" t="n">
-        <v>790283</v>
+        <v>789423</v>
       </c>
       <c r="I44" t="n">
-        <v>8.140000000000001</v>
+        <v>186.49</v>
       </c>
       <c r="J44" t="n">
-        <v>12.53</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>148816</v>
+        <v>106348</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
@@ -2147,13 +2147,203 @@
         <v>46259</v>
       </c>
       <c r="H45" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>11.29</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>125</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H46" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I46" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="J46" t="n">
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>96</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SILAS SALVIANO PRATI</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>142645</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>25E17F</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G47" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H47" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I47" t="n">
+        <v>81.64</v>
+      </c>
+      <c r="J47" t="n">
+        <v>81.64</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>39</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G48" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H48" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I48" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J48" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>147</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G49" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H49" t="n">
         <v>33928</v>
       </c>
-      <c r="I45" t="n">
+      <c r="I49" t="n">
         <v>10.43</v>
       </c>
-      <c r="J45" t="n">
+      <c r="J49" t="n">
         <v>10.43</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>39</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>157761</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>4O4518</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>46357</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H50" t="n">
+        <v>790808</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>104.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:30:04
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1285,39 +1285,39 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>152839</v>
+        <v>139865</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>5582</v>
+        <v>794365</v>
       </c>
       <c r="I23" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>80.55</v>
+        <v>48.02</v>
       </c>
     </row>
     <row r="24">
@@ -1335,163 +1335,163 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>154122</v>
+        <v>152839</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>794919</v>
+        <v>5582</v>
       </c>
       <c r="I24" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
       <c r="J24" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>155008</v>
+        <v>154122</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>790283</v>
+        <v>794919</v>
       </c>
       <c r="I25" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
       <c r="J25" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>155969</v>
+        <v>155008</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>789423</v>
+        <v>790283</v>
       </c>
       <c r="I26" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
       <c r="J26" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>110370</v>
+        <v>155969</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I27" t="n">
-        <v>62.52</v>
+        <v>510.49</v>
       </c>
       <c r="J27" t="n">
-        <v>62.52</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>142124</v>
+        <v>110370</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -1501,35 +1501,35 @@
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I28" t="n">
-        <v>185.14</v>
+        <v>62.52</v>
       </c>
       <c r="J28" t="n">
-        <v>185.13</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>147194</v>
+        <v>142124</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
@@ -1539,13 +1539,13 @@
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I29" t="n">
-        <v>7.99</v>
+        <v>185.14</v>
       </c>
       <c r="J29" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="30">
@@ -1563,24 +1563,24 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>148828</v>
+        <v>147194</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>792019</v>
+        <v>33928</v>
       </c>
       <c r="I30" t="n">
-        <v>93.70999999999999</v>
+        <v>7.99</v>
       </c>
       <c r="J30" t="n">
         <v>0</v>
@@ -1589,23 +1589,23 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>155970</v>
+        <v>148828</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -1615,89 +1615,89 @@
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>789423</v>
+        <v>792019</v>
       </c>
       <c r="I31" t="n">
-        <v>283.62</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J31" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>81973</v>
+        <v>155970</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I32" t="n">
-        <v>6.24</v>
+        <v>283.62</v>
       </c>
       <c r="J32" t="n">
-        <v>6.24</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>142672</v>
+        <v>81973</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I33" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
       <c r="J33" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="34">
@@ -1707,61 +1707,61 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>142886</v>
+        <v>142672</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I34" t="n">
-        <v>65.23999999999999</v>
+        <v>39.31</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>53</v>
+        <v>111</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>153194</v>
+        <v>142886</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
@@ -1770,7 +1770,7 @@
         <v>789423</v>
       </c>
       <c r="I35" t="n">
-        <v>155.28</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1779,27 +1779,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>155919</v>
+        <v>153194</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46259</v>
@@ -1808,86 +1808,86 @@
         <v>789423</v>
       </c>
       <c r="I36" t="n">
-        <v>158.77</v>
+        <v>155.28</v>
       </c>
       <c r="J36" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>159083</v>
+        <v>155919</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
       <c r="J37" t="n">
-        <v>88.59999999999999</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>58</v>
+        <v>125</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>66958</v>
+        <v>159083</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>789525</v>
+        <v>794365</v>
       </c>
       <c r="I38" t="n">
-        <v>59.39</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>59.39</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="39">
@@ -1897,222 +1897,222 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>92720</v>
+        <v>55476</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>37273</v>
+        <v>30791</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>6.88</v>
+        <v>56.83</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>140760</v>
+        <v>66958</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>789423</v>
+        <v>789525</v>
       </c>
       <c r="I40" t="n">
-        <v>37.39</v>
+        <v>59.39</v>
       </c>
       <c r="J40" t="n">
-        <v>37.39</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>49964</v>
+        <v>92720</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>789228</v>
+        <v>37273</v>
       </c>
       <c r="I41" t="n">
-        <v>82.8</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>147</v>
+        <v>111</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>84824</v>
+        <v>140760</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H42" t="n">
-        <v>789662</v>
+        <v>789423</v>
       </c>
       <c r="I42" t="n">
-        <v>27.31</v>
+        <v>37.39</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>88358</v>
+        <v>49964</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>793056</v>
+        <v>789228</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>82.8</v>
       </c>
       <c r="J43" t="n">
-        <v>21.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>105546</v>
+        <v>55204</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H44" t="n">
-        <v>789423</v>
+        <v>30791</v>
       </c>
       <c r="I44" t="n">
-        <v>186.49</v>
+        <v>43.88</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
@@ -2121,39 +2121,39 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>106348</v>
+        <v>84824</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>65455</v>
+        <v>789662</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>27.31</v>
       </c>
       <c r="J45" t="n">
-        <v>11.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -2171,11 +2171,11 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>106364</v>
+        <v>88358</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -2185,51 +2185,51 @@
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>65455</v>
+        <v>793056</v>
       </c>
       <c r="I46" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>51.35</v>
+        <v>21.4</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>142645</v>
+        <v>105546</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>789429</v>
+        <v>789423</v>
       </c>
       <c r="I47" t="n">
-        <v>81.64</v>
+        <v>186.49</v>
       </c>
       <c r="J47" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -2247,102 +2247,216 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>146095</v>
+        <v>106348</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>790283</v>
+        <v>65455</v>
       </c>
       <c r="I48" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>20.67</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>148816</v>
+        <v>106364</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>33928</v>
+        <v>65455</v>
       </c>
       <c r="I49" t="n">
-        <v>10.43</v>
+        <v>51.35</v>
       </c>
       <c r="J49" t="n">
-        <v>10.43</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>96</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>SILAS SALVIANO PRATI</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>142645</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>25E17F</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G50" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H50" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I50" t="n">
+        <v>81.64</v>
+      </c>
+      <c r="J50" t="n">
+        <v>81.64</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>PI</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B51" t="n">
         <v>39</v>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D51" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G51" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H51" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I51" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J51" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>147</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H52" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I52" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J52" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>39</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
         <v>157761</v>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F53" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G50" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H50" t="n">
+      <c r="G53" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H53" t="n">
         <v>790808</v>
       </c>
-      <c r="I50" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" t="n">
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 15:45:02
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -867,61 +867,61 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>139865</v>
+        <v>79995</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>B25B2383</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H12" t="n">
-        <v>794365</v>
+        <v>47252</v>
       </c>
       <c r="I12" t="n">
-        <v>25.42</v>
+        <v>144.41</v>
       </c>
       <c r="J12" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>142466</v>
+        <v>139865</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>25I07B</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -931,51 +931,51 @@
         <v>46259</v>
       </c>
       <c r="H13" t="n">
-        <v>789429</v>
+        <v>794365</v>
       </c>
       <c r="I13" t="n">
-        <v>39.97</v>
+        <v>25.42</v>
       </c>
       <c r="J13" t="n">
-        <v>457.31</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>155114</v>
+        <v>142466</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0000267854</t>
+          <t>25I07B</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46327</v>
+        <v>46419</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H14" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I14" t="n">
-        <v>84.31</v>
+        <v>39.97</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>457.31</v>
       </c>
     </row>
     <row r="15">
@@ -985,35 +985,35 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>98663</v>
+        <v>155114</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>4R6305</t>
+          <t>0000267854</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46447</v>
+        <v>46327</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H15" t="n">
-        <v>37273</v>
+        <v>789423</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>84.31</v>
       </c>
       <c r="J15" t="n">
-        <v>29.51</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1023,73 +1023,73 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>115223</v>
+        <v>98663</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H16" t="n">
-        <v>789423</v>
+        <v>37273</v>
       </c>
       <c r="I16" t="n">
-        <v>62.07</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>62.07</v>
       </c>
       <c r="J17" t="n">
-        <v>346.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -1099,95 +1099,95 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>153462</v>
+        <v>118036</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>30791</v>
+        <v>790808</v>
       </c>
       <c r="I18" t="n">
-        <v>1302.28</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>158962</v>
+        <v>153462</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="I19" t="n">
-        <v>196.61</v>
+        <v>1302.28</v>
       </c>
       <c r="J19" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>20206</v>
+        <v>158962</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>PR1365</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
@@ -1197,225 +1197,225 @@
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="I20" t="n">
-        <v>33.94</v>
+        <v>196.61</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>64130</v>
+        <v>20206</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>45870</v>
+        <v>46508</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>33.96</v>
       </c>
       <c r="J21" t="n">
-        <v>118.94</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>120901</v>
+        <v>64130</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46327</v>
+        <v>45870</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>33057</v>
+        <v>30791</v>
       </c>
       <c r="I22" t="n">
-        <v>81.26000000000001</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>118.94</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>139865</v>
+        <v>120901</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>794365</v>
+        <v>33057</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J23" t="n">
-        <v>48.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>152839</v>
+        <v>123315</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>65651413</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>5582</v>
+        <v>30791</v>
       </c>
       <c r="I24" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>80.55</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>154122</v>
+        <v>139865</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>794919</v>
+        <v>794365</v>
       </c>
       <c r="I25" t="n">
-        <v>150.95</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>150.95</v>
+        <v>68.62</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>155008</v>
+        <v>152839</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1425,13 +1425,13 @@
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>790283</v>
+        <v>5582</v>
       </c>
       <c r="I26" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
       <c r="J26" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="27">
@@ -1449,27 +1449,27 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>155969</v>
+        <v>154122</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>789423</v>
+        <v>794919</v>
       </c>
       <c r="I27" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
       <c r="J27" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="28">
@@ -1487,11 +1487,11 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>110370</v>
+        <v>155008</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -1501,13 +1501,13 @@
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>47252</v>
+        <v>790283</v>
       </c>
       <c r="I28" t="n">
-        <v>62.52</v>
+        <v>18.72</v>
       </c>
       <c r="J28" t="n">
-        <v>62.52</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="29">
@@ -1525,100 +1525,100 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>142124</v>
+        <v>155969</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>31305</v>
+        <v>789423</v>
       </c>
       <c r="I29" t="n">
-        <v>185.14</v>
+        <v>510.49</v>
       </c>
       <c r="J29" t="n">
-        <v>185.13</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>147194</v>
+        <v>55476</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46388</v>
+        <v>46478</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>33928</v>
+        <v>30791</v>
       </c>
       <c r="I30" t="n">
-        <v>7.99</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>148828</v>
+        <v>79987</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>792019</v>
+        <v>47252</v>
       </c>
       <c r="I31" t="n">
-        <v>93.70999999999999</v>
+        <v>111.1</v>
       </c>
       <c r="J31" t="n">
         <v>0</v>
@@ -1627,150 +1627,150 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>155970</v>
+        <v>110370</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I32" t="n">
-        <v>283.62</v>
+        <v>62.52</v>
       </c>
       <c r="J32" t="n">
-        <v>283.62</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>81973</v>
+        <v>142124</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>47252</v>
+        <v>31305</v>
       </c>
       <c r="I33" t="n">
-        <v>6.24</v>
+        <v>185.14</v>
       </c>
       <c r="J33" t="n">
-        <v>6.24</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>142672</v>
+        <v>147194</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>789429</v>
+        <v>33928</v>
       </c>
       <c r="I34" t="n">
-        <v>39.31</v>
+        <v>7.99</v>
       </c>
       <c r="J34" t="n">
-        <v>39.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>142886</v>
+        <v>148828</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>789423</v>
+        <v>792019</v>
       </c>
       <c r="I35" t="n">
-        <v>65.23999999999999</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -1779,23 +1779,23 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>153194</v>
+        <v>155970</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -1808,48 +1808,48 @@
         <v>789423</v>
       </c>
       <c r="I36" t="n">
-        <v>155.28</v>
+        <v>283.62</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>155919</v>
+        <v>81973</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I37" t="n">
-        <v>158.77</v>
+        <v>6.24</v>
       </c>
       <c r="J37" t="n">
-        <v>158.77</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="38">
@@ -1859,35 +1859,35 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>159083</v>
+        <v>102393</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>794365</v>
+        <v>53333</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>88.59999999999999</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="39">
@@ -1897,95 +1897,95 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>55476</v>
+        <v>142672</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>30791</v>
+        <v>789429</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
       <c r="J39" t="n">
-        <v>56.83</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>58</v>
+        <v>111</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>66958</v>
+        <v>142886</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>789525</v>
+        <v>789423</v>
       </c>
       <c r="I40" t="n">
-        <v>59.39</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J40" t="n">
-        <v>59.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>92720</v>
+        <v>153194</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -1995,39 +1995,39 @@
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>37273</v>
+        <v>789423</v>
       </c>
       <c r="I41" t="n">
-        <v>0</v>
+        <v>155.28</v>
       </c>
       <c r="J41" t="n">
-        <v>6.88</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>140760</v>
+        <v>155919</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
@@ -2036,74 +2036,74 @@
         <v>789423</v>
       </c>
       <c r="I42" t="n">
-        <v>37.39</v>
+        <v>158.77</v>
       </c>
       <c r="J42" t="n">
-        <v>37.39</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>49964</v>
+        <v>159083</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>789228</v>
+        <v>794365</v>
       </c>
       <c r="I43" t="n">
-        <v>82.8</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>55204</v>
+        <v>55476</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
@@ -2112,48 +2112,48 @@
         <v>30791</v>
       </c>
       <c r="I44" t="n">
-        <v>43.88</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>56.83</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>147</v>
+        <v>58</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>84824</v>
+        <v>66958</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>789662</v>
+        <v>789525</v>
       </c>
       <c r="I45" t="n">
-        <v>27.31</v>
+        <v>59.39</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="46">
@@ -2171,11 +2171,11 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>88358</v>
+        <v>92720</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -2185,35 +2185,35 @@
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>793056</v>
+        <v>37273</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>21.4</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>53</v>
+        <v>120</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>105546</v>
+        <v>100471</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -2223,10 +2223,10 @@
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I47" t="n">
-        <v>186.49</v>
+        <v>126.06</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
@@ -2235,39 +2235,39 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>106348</v>
+        <v>140760</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>65455</v>
+        <v>789423</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
       <c r="J48" t="n">
-        <v>11.29</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="49">
@@ -2285,91 +2285,91 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>106364</v>
+        <v>145507</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46508</v>
+        <v>46485</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>65455</v>
+        <v>47252</v>
       </c>
       <c r="I49" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>51.35</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>142645</v>
+        <v>160073</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H50" t="n">
-        <v>789429</v>
+        <v>795751</v>
       </c>
       <c r="I50" t="n">
-        <v>81.64</v>
+        <v>74.92</v>
       </c>
       <c r="J50" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>146095</v>
+        <v>44733</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46508</v>
+        <v>46113</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46259</v>
@@ -2378,48 +2378,48 @@
         <v>790283</v>
       </c>
       <c r="I51" t="n">
-        <v>8.15</v>
+        <v>27.55</v>
       </c>
       <c r="J51" t="n">
-        <v>20.67</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>148816</v>
+        <v>49964</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46478</v>
+        <v>46419</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>33928</v>
+        <v>789228</v>
       </c>
       <c r="I52" t="n">
-        <v>10.43</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J52" t="n">
-        <v>10.43</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="53">
@@ -2437,26 +2437,406 @@
         </is>
       </c>
       <c r="D53" t="n">
+        <v>55204</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>08681216</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G53" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H53" t="n">
+        <v>30791</v>
+      </c>
+      <c r="I53" t="n">
+        <v>43.92</v>
+      </c>
+      <c r="J53" t="n">
+        <v>43.92</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>147</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>84824</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FKP06475</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H54" t="n">
+        <v>789662</v>
+      </c>
+      <c r="I54" t="n">
+        <v>27.31</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>125</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>88358</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>GRA01137</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H55" t="n">
+        <v>793056</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>42.8</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>53</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>105546</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>0000270940</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="n">
+        <v>46419</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H56" t="n">
+        <v>789423</v>
+      </c>
+      <c r="I56" t="n">
+        <v>186.49</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>39</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>106348</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>BR181245</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G57" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H57" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>11.29</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>125</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H58" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I58" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="J58" t="n">
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>96</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>SILAS SALVIANO PRATI</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>142645</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>25E17F</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G59" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H59" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I59" t="n">
+        <v>81.64</v>
+      </c>
+      <c r="J59" t="n">
+        <v>81.64</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>39</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H60" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I60" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J60" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>147</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G61" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H61" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I61" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J61" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>39</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H62" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I62" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>39</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
         <v>157761</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F53" s="2" t="n">
+      <c r="F63" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G53" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H53" t="n">
+      <c r="G63" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H63" t="n">
         <v>790808</v>
       </c>
-      <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="n">
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:00:04
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1057,36 +1057,36 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>115223</v>
+        <v>110264</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>B25B0673</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I17" t="n">
-        <v>62.07</v>
+        <v>9.35</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1095,39 +1095,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>62.07</v>
       </c>
       <c r="J18" t="n">
-        <v>346.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1137,95 +1137,95 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>153462</v>
+        <v>118036</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>30791</v>
+        <v>790808</v>
       </c>
       <c r="I19" t="n">
-        <v>1302.28</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>158962</v>
+        <v>153462</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="I20" t="n">
-        <v>196.61</v>
+        <v>1302.28</v>
       </c>
       <c r="J20" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>20206</v>
+        <v>158962</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PR1365</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
@@ -1235,127 +1235,127 @@
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="I21" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
       <c r="J21" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>64130</v>
+        <v>20206</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>45870</v>
+        <v>46508</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>33.96</v>
       </c>
       <c r="J22" t="n">
-        <v>118.94</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>120901</v>
+        <v>64130</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>46327</v>
+        <v>45870</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>33057</v>
+        <v>30791</v>
       </c>
       <c r="I23" t="n">
-        <v>81.26000000000001</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>476.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>123315</v>
+        <v>120901</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>65651413</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J24" t="n">
-        <v>24.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -1373,11 +1373,11 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>139865</v>
+        <v>123315</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>65651413</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
@@ -1387,51 +1387,51 @@
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>794365</v>
+        <v>30791</v>
       </c>
       <c r="I25" t="n">
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>68.62</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>152839</v>
+        <v>139865</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>5582</v>
+        <v>794365</v>
       </c>
       <c r="I26" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>80.55</v>
+        <v>68.62</v>
       </c>
     </row>
     <row r="27">
@@ -1449,217 +1449,217 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>154122</v>
+        <v>152839</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>794919</v>
+        <v>5582</v>
       </c>
       <c r="I27" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
       <c r="J27" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>155008</v>
+        <v>154122</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>790283</v>
+        <v>794919</v>
       </c>
       <c r="I28" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
       <c r="J28" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>155969</v>
+        <v>155008</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>789423</v>
+        <v>790283</v>
       </c>
       <c r="I29" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
       <c r="J29" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>55476</v>
+        <v>155969</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>510.49</v>
       </c>
       <c r="J30" t="n">
-        <v>56.86</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>79987</v>
+        <v>55476</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>B25B1713</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I31" t="n">
-        <v>111.1</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>110370</v>
+        <v>64130</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46388</v>
+        <v>45870</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I32" t="n">
-        <v>62.52</v>
+        <v>59.5</v>
       </c>
       <c r="J32" t="n">
-        <v>62.52</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="33">
@@ -1677,27 +1677,27 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>142124</v>
+        <v>79987</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I33" t="n">
-        <v>185.14</v>
+        <v>111.1</v>
       </c>
       <c r="J33" t="n">
-        <v>185.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -1715,11 +1715,11 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>147194</v>
+        <v>110370</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
@@ -1729,89 +1729,89 @@
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I34" t="n">
-        <v>7.99</v>
+        <v>62.52</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>148828</v>
+        <v>142124</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>792019</v>
+        <v>31305</v>
       </c>
       <c r="I35" t="n">
-        <v>93.70999999999999</v>
+        <v>185.14</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>155970</v>
+        <v>147194</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I36" t="n">
-        <v>283.62</v>
+        <v>7.99</v>
       </c>
       <c r="J36" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -1829,103 +1829,103 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>81973</v>
+        <v>148828</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>47252</v>
+        <v>792019</v>
       </c>
       <c r="I37" t="n">
-        <v>6.24</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J37" t="n">
-        <v>6.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>102393</v>
+        <v>155970</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>4O3174</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46357</v>
+        <v>46508</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>53333</v>
+        <v>789423</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>283.62</v>
       </c>
       <c r="J38" t="n">
-        <v>2.02</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>142672</v>
+        <v>81973</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I39" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
       <c r="J39" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="40">
@@ -1935,57 +1935,57 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>142886</v>
+        <v>102393</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I40" t="n">
-        <v>65.23999999999999</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>153194</v>
+        <v>142672</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -1995,35 +1995,35 @@
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I41" t="n">
-        <v>155.28</v>
+        <v>39.31</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>155919</v>
+        <v>142886</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
@@ -2036,124 +2036,124 @@
         <v>789423</v>
       </c>
       <c r="I42" t="n">
-        <v>158.77</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J42" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>159083</v>
+        <v>153194</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>155.28</v>
       </c>
       <c r="J43" t="n">
-        <v>88.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>55476</v>
+        <v>155919</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H44" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
       <c r="J44" t="n">
-        <v>56.83</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>58</v>
+        <v>125</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>66958</v>
+        <v>159083</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>789525</v>
+        <v>794365</v>
       </c>
       <c r="I45" t="n">
-        <v>59.39</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>59.39</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="46">
@@ -2163,35 +2163,35 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>92720</v>
+        <v>55476</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>37273</v>
+        <v>30791</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>6.88</v>
+        <v>56.83</v>
       </c>
     </row>
     <row r="47">
@@ -2201,35 +2201,35 @@
         </is>
       </c>
       <c r="B47" t="n">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>100471</v>
+        <v>66958</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>4P2788</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>53333</v>
+        <v>789525</v>
       </c>
       <c r="I47" t="n">
-        <v>126.06</v>
+        <v>59.39</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="48">
@@ -2239,95 +2239,95 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>140760</v>
+        <v>92720</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>789423</v>
+        <v>37273</v>
       </c>
       <c r="I48" t="n">
-        <v>37.39</v>
+        <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>37.39</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>145507</v>
+        <v>100471</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46485</v>
+        <v>46419</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
+        <v>126.28</v>
       </c>
       <c r="J49" t="n">
-        <v>26.34</v>
+        <v>126.28</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>160073</v>
+        <v>140760</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
@@ -2337,51 +2337,51 @@
         <v>46259</v>
       </c>
       <c r="H50" t="n">
-        <v>795751</v>
+        <v>789423</v>
       </c>
       <c r="I50" t="n">
-        <v>74.92</v>
+        <v>37.39</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>44733</v>
+        <v>145507</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46113</v>
+        <v>46485</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H51" t="n">
-        <v>790283</v>
+        <v>47252</v>
       </c>
       <c r="I51" t="n">
-        <v>27.55</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>27.55</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="52">
@@ -2399,176 +2399,176 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>49964</v>
+        <v>160073</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>789228</v>
+        <v>795751</v>
       </c>
       <c r="I52" t="n">
-        <v>82.84999999999999</v>
+        <v>74.92</v>
       </c>
       <c r="J52" t="n">
-        <v>82.84999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>55204</v>
+        <v>44733</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46447</v>
+        <v>46113</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H53" t="n">
-        <v>30791</v>
+        <v>790283</v>
       </c>
       <c r="I53" t="n">
-        <v>43.92</v>
+        <v>27.55</v>
       </c>
       <c r="J53" t="n">
-        <v>43.92</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>84824</v>
+        <v>49964</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H54" t="n">
-        <v>789662</v>
+        <v>789228</v>
       </c>
       <c r="I54" t="n">
-        <v>27.31</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>88358</v>
+        <v>55204</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H55" t="n">
-        <v>793056</v>
+        <v>30791</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>43.92</v>
       </c>
       <c r="J55" t="n">
-        <v>42.8</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>53</v>
+        <v>147</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>105546</v>
+        <v>84824</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H56" t="n">
-        <v>789423</v>
+        <v>789662</v>
       </c>
       <c r="I56" t="n">
-        <v>186.49</v>
+        <v>27.31</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -2577,137 +2577,137 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>106348</v>
+        <v>88358</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H57" t="n">
-        <v>65455</v>
+        <v>793056</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
       </c>
       <c r="J57" t="n">
-        <v>11.29</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>106364</v>
+        <v>105546</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H58" t="n">
-        <v>65455</v>
+        <v>789423</v>
       </c>
       <c r="I58" t="n">
-        <v>51.35</v>
+        <v>186.49</v>
       </c>
       <c r="J58" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>142645</v>
+        <v>106348</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H59" t="n">
-        <v>789429</v>
+        <v>65455</v>
       </c>
       <c r="I59" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>81.64</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>146095</v>
+        <v>106364</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
@@ -2717,51 +2717,51 @@
         <v>46259</v>
       </c>
       <c r="H60" t="n">
-        <v>790283</v>
+        <v>65455</v>
       </c>
       <c r="I60" t="n">
-        <v>8.15</v>
+        <v>51.35</v>
       </c>
       <c r="J60" t="n">
-        <v>20.67</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>147</v>
+        <v>96</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>148816</v>
+        <v>142645</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>25E17F</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H61" t="n">
-        <v>33928</v>
+        <v>789429</v>
       </c>
       <c r="I61" t="n">
-        <v>10.43</v>
+        <v>81.64</v>
       </c>
       <c r="J61" t="n">
-        <v>10.43</v>
+        <v>81.64</v>
       </c>
     </row>
     <row r="62">
@@ -2779,64 +2779,140 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>148823</v>
+        <v>146095</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>252535</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H62" t="n">
-        <v>33928</v>
+        <v>790283</v>
       </c>
       <c r="I62" t="n">
-        <v>53.82</v>
+        <v>8.15</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>147</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G63" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H63" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I63" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J63" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>PI</t>
         </is>
       </c>
-      <c r="B63" t="n">
+      <c r="B64" t="n">
         <v>39</v>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
-      <c r="D63" t="n">
+      <c r="D64" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H64" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I64" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>39</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
         <v>157761</v>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F63" s="2" t="n">
+      <c r="F65" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G63" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H63" t="n">
+      <c r="G65" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H65" t="n">
         <v>790808</v>
       </c>
-      <c r="I63" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" t="n">
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:15:02
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1057,36 +1057,36 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>110264</v>
+        <v>102024</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>B25B0673</t>
+          <t>4P0969</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I17" t="n">
-        <v>9.35</v>
+        <v>18.67</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1095,36 +1095,36 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>115223</v>
+        <v>110264</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>B25B0673</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I18" t="n">
-        <v>62.07</v>
+        <v>9.35</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1133,39 +1133,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>62.07</v>
       </c>
       <c r="J19" t="n">
-        <v>346.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -1175,95 +1175,95 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>153462</v>
+        <v>118036</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>30791</v>
+        <v>790808</v>
       </c>
       <c r="I20" t="n">
-        <v>1302.28</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>158962</v>
+        <v>153462</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="I21" t="n">
-        <v>196.61</v>
+        <v>1302.28</v>
       </c>
       <c r="J21" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>20206</v>
+        <v>158962</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PR1365</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -1273,127 +1273,127 @@
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="I22" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
       <c r="J22" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>64130</v>
+        <v>20206</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>45870</v>
+        <v>46508</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>33.96</v>
       </c>
       <c r="J23" t="n">
-        <v>476.1</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>120901</v>
+        <v>64130</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46327</v>
+        <v>45870</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>33057</v>
+        <v>30791</v>
       </c>
       <c r="I24" t="n">
-        <v>81.26000000000001</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>476.1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>123315</v>
+        <v>120901</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>65651413</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J25" t="n">
-        <v>24.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -1411,11 +1411,11 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>139865</v>
+        <v>123315</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>65651413</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1425,51 +1425,51 @@
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>794365</v>
+        <v>30791</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>68.62</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>152839</v>
+        <v>139865</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>5582</v>
+        <v>794365</v>
       </c>
       <c r="I27" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>80.55</v>
+        <v>68.62</v>
       </c>
     </row>
     <row r="28">
@@ -1487,167 +1487,167 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>154122</v>
+        <v>152839</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>794919</v>
+        <v>5582</v>
       </c>
       <c r="I28" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
       <c r="J28" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>155008</v>
+        <v>154122</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>790283</v>
+        <v>794919</v>
       </c>
       <c r="I29" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
       <c r="J29" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>155969</v>
+        <v>155008</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>789423</v>
+        <v>790283</v>
       </c>
       <c r="I30" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
       <c r="J30" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>55476</v>
+        <v>155969</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>510.49</v>
       </c>
       <c r="J31" t="n">
-        <v>56.86</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>64130</v>
+        <v>55476</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>45870</v>
+        <v>46478</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
@@ -1656,74 +1656,74 @@
         <v>30791</v>
       </c>
       <c r="I32" t="n">
-        <v>59.5</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>59.5</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>79987</v>
+        <v>64130</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>B25B1713</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46447</v>
+        <v>45870</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I33" t="n">
-        <v>111.1</v>
+        <v>59.5</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>110370</v>
+        <v>79987</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
@@ -1732,32 +1732,32 @@
         <v>47252</v>
       </c>
       <c r="I34" t="n">
-        <v>62.52</v>
+        <v>111.1</v>
       </c>
       <c r="J34" t="n">
-        <v>62.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>142124</v>
+        <v>110370</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -1767,35 +1767,35 @@
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I35" t="n">
-        <v>185.14</v>
+        <v>62.52</v>
       </c>
       <c r="J35" t="n">
-        <v>185.13</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>147194</v>
+        <v>142124</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -1805,13 +1805,13 @@
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I36" t="n">
-        <v>7.99</v>
+        <v>185.14</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="37">
@@ -1829,24 +1829,24 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>148828</v>
+        <v>147194</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>792019</v>
+        <v>33928</v>
       </c>
       <c r="I37" t="n">
-        <v>93.70999999999999</v>
+        <v>7.99</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1855,23 +1855,23 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>155970</v>
+        <v>148828</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -1881,13 +1881,13 @@
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>789423</v>
+        <v>792019</v>
       </c>
       <c r="I38" t="n">
-        <v>283.62</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J38" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -1897,111 +1897,111 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>81973</v>
+        <v>153194</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>0000293059</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I39" t="n">
-        <v>6.24</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="J39" t="n">
-        <v>6.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>102393</v>
+        <v>155970</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>4O3174</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46357</v>
+        <v>46508</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>53333</v>
+        <v>789423</v>
       </c>
       <c r="I40" t="n">
-        <v>0</v>
+        <v>283.62</v>
       </c>
       <c r="J40" t="n">
-        <v>2.02</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>142672</v>
+        <v>81973</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I41" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
       <c r="J41" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="42">
@@ -2011,57 +2011,57 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>142886</v>
+        <v>102393</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H42" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I42" t="n">
-        <v>65.23999999999999</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>153194</v>
+        <v>142672</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
@@ -2071,35 +2071,35 @@
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I43" t="n">
-        <v>155.28</v>
+        <v>39.31</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>155919</v>
+        <v>142886</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
@@ -2112,124 +2112,124 @@
         <v>789423</v>
       </c>
       <c r="I44" t="n">
-        <v>158.77</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J44" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>159083</v>
+        <v>153194</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>155.28</v>
       </c>
       <c r="J45" t="n">
-        <v>88.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>55476</v>
+        <v>155919</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
       <c r="J46" t="n">
-        <v>56.83</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>58</v>
+        <v>125</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>66958</v>
+        <v>159083</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>789525</v>
+        <v>794365</v>
       </c>
       <c r="I47" t="n">
-        <v>59.39</v>
+        <v>0</v>
       </c>
       <c r="J47" t="n">
-        <v>59.39</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="48">
@@ -2239,35 +2239,35 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>92720</v>
+        <v>55476</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>37273</v>
+        <v>30791</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>6.88</v>
+        <v>56.83</v>
       </c>
     </row>
     <row r="49">
@@ -2277,35 +2277,35 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>100471</v>
+        <v>66958</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>4P2788</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>53333</v>
+        <v>789525</v>
       </c>
       <c r="I49" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
       <c r="J49" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="50">
@@ -2315,95 +2315,95 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>140760</v>
+        <v>92720</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H50" t="n">
-        <v>789423</v>
+        <v>37273</v>
       </c>
       <c r="I50" t="n">
-        <v>37.39</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>37.39</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>145507</v>
+        <v>100471</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46485</v>
+        <v>46419</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H51" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>126.28</v>
       </c>
       <c r="J51" t="n">
-        <v>26.34</v>
+        <v>126.28</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>160073</v>
+        <v>140760</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
@@ -2413,51 +2413,51 @@
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>795751</v>
+        <v>789423</v>
       </c>
       <c r="I52" t="n">
-        <v>74.92</v>
+        <v>37.39</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>44733</v>
+        <v>145507</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46113</v>
+        <v>46485</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H53" t="n">
-        <v>790283</v>
+        <v>47252</v>
       </c>
       <c r="I53" t="n">
-        <v>27.55</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>27.55</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="54">
@@ -2475,176 +2475,176 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>49964</v>
+        <v>160073</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H54" t="n">
-        <v>789228</v>
+        <v>795751</v>
       </c>
       <c r="I54" t="n">
-        <v>82.84999999999999</v>
+        <v>74.92</v>
       </c>
       <c r="J54" t="n">
-        <v>82.84999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>55204</v>
+        <v>44733</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>46447</v>
+        <v>46113</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H55" t="n">
-        <v>30791</v>
+        <v>790283</v>
       </c>
       <c r="I55" t="n">
-        <v>43.92</v>
+        <v>27.55</v>
       </c>
       <c r="J55" t="n">
-        <v>43.92</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>84824</v>
+        <v>49964</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H56" t="n">
-        <v>789662</v>
+        <v>789228</v>
       </c>
       <c r="I56" t="n">
-        <v>27.31</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J56" t="n">
-        <v>0</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>88358</v>
+        <v>55204</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H57" t="n">
-        <v>793056</v>
+        <v>30791</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
+        <v>43.92</v>
       </c>
       <c r="J57" t="n">
-        <v>42.8</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>53</v>
+        <v>147</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>105546</v>
+        <v>84824</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H58" t="n">
-        <v>789423</v>
+        <v>789662</v>
       </c>
       <c r="I58" t="n">
-        <v>186.49</v>
+        <v>27.31</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -2653,61 +2653,61 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>106348</v>
+        <v>88358</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H59" t="n">
-        <v>65455</v>
+        <v>793056</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>11.29</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>106364</v>
+        <v>101583</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>4V6234</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
@@ -2717,51 +2717,51 @@
         <v>46259</v>
       </c>
       <c r="H60" t="n">
-        <v>65455</v>
+        <v>53333</v>
       </c>
       <c r="I60" t="n">
-        <v>51.35</v>
+        <v>125.05</v>
       </c>
       <c r="J60" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>142645</v>
+        <v>105546</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H61" t="n">
-        <v>789429</v>
+        <v>789423</v>
       </c>
       <c r="I61" t="n">
-        <v>81.64</v>
+        <v>186.49</v>
       </c>
       <c r="J61" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -2779,103 +2779,103 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>146095</v>
+        <v>106348</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H62" t="n">
-        <v>790283</v>
+        <v>65455</v>
       </c>
       <c r="I62" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>20.67</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>148816</v>
+        <v>106364</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H63" t="n">
-        <v>33928</v>
+        <v>65455</v>
       </c>
       <c r="I63" t="n">
-        <v>10.43</v>
+        <v>51.35</v>
       </c>
       <c r="J63" t="n">
-        <v>10.43</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>148823</v>
+        <v>142645</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>25E17F</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H64" t="n">
-        <v>33928</v>
+        <v>789429</v>
       </c>
       <c r="I64" t="n">
-        <v>53.82</v>
+        <v>81.64</v>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>81.64</v>
       </c>
     </row>
     <row r="65">
@@ -2893,26 +2893,140 @@
         </is>
       </c>
       <c r="D65" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G65" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H65" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I65" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J65" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>147</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H66" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I66" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J66" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>39</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G67" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H67" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I67" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>39</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
         <v>157761</v>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F65" s="2" t="n">
+      <c r="F68" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G65" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H65" t="n">
+      <c r="G68" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H68" t="n">
         <v>790808</v>
       </c>
-      <c r="I65" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" t="n">
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:30:04
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1031,100 +1031,100 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>98663</v>
+        <v>95052</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>4R6305</t>
+          <t>570950</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H16" t="n">
-        <v>37273</v>
+        <v>47252</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>29.51</v>
+        <v>312.35</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>102024</v>
+        <v>98663</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4P0969</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46357</v>
+        <v>46447</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>53333</v>
+        <v>37273</v>
       </c>
       <c r="I17" t="n">
-        <v>18.67</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>0</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>110264</v>
+        <v>102024</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>B25B0673</t>
+          <t>4P0969</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I18" t="n">
-        <v>9.35</v>
+        <v>18.67</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -1133,36 +1133,36 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>115223</v>
+        <v>110264</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>B25B0673</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I19" t="n">
-        <v>62.07</v>
+        <v>9.35</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1171,39 +1171,39 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>62.07</v>
       </c>
       <c r="J20" t="n">
-        <v>346.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -1213,95 +1213,95 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>153462</v>
+        <v>118036</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>30791</v>
+        <v>790808</v>
       </c>
       <c r="I21" t="n">
-        <v>1302.28</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>158962</v>
+        <v>153462</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="I22" t="n">
-        <v>196.61</v>
+        <v>1302.28</v>
       </c>
       <c r="J22" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>20206</v>
+        <v>158962</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PR1365</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1311,127 +1311,127 @@
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="I23" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
       <c r="J23" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>64130</v>
+        <v>20206</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>45870</v>
+        <v>46508</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>33.96</v>
       </c>
       <c r="J24" t="n">
-        <v>476.1</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>120901</v>
+        <v>64130</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>46327</v>
+        <v>45870</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>33057</v>
+        <v>30791</v>
       </c>
       <c r="I25" t="n">
-        <v>81.26000000000001</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>0</v>
+        <v>476.1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>123315</v>
+        <v>120901</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>65651413</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>30791</v>
+        <v>33057</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J26" t="n">
-        <v>24.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -1449,11 +1449,11 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>139865</v>
+        <v>123315</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>65651413</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -1463,51 +1463,51 @@
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>794365</v>
+        <v>30791</v>
       </c>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>68.62</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>152839</v>
+        <v>139865</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>5582</v>
+        <v>794365</v>
       </c>
       <c r="I28" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>80.55</v>
+        <v>117.18</v>
       </c>
     </row>
     <row r="29">
@@ -1525,167 +1525,167 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>154122</v>
+        <v>152839</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>794919</v>
+        <v>5582</v>
       </c>
       <c r="I29" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
       <c r="J29" t="n">
-        <v>150.95</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>155008</v>
+        <v>154122</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>790283</v>
+        <v>794919</v>
       </c>
       <c r="I30" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
       <c r="J30" t="n">
-        <v>18.72</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>155969</v>
+        <v>155008</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>789423</v>
+        <v>790283</v>
       </c>
       <c r="I31" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
       <c r="J31" t="n">
-        <v>510.49</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>55476</v>
+        <v>155969</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>510.49</v>
       </c>
       <c r="J32" t="n">
-        <v>56.86</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>64130</v>
+        <v>55476</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>45870</v>
+        <v>46478</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
@@ -1694,159 +1694,159 @@
         <v>30791</v>
       </c>
       <c r="I33" t="n">
-        <v>59.5</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>59.5</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>79987</v>
+        <v>55476</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>B25B1713</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I34" t="n">
-        <v>111.1</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>113.71</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>110370</v>
+        <v>64130</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46388</v>
+        <v>45870</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I35" t="n">
-        <v>62.52</v>
+        <v>59.5</v>
       </c>
       <c r="J35" t="n">
-        <v>62.52</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>142124</v>
+        <v>66958</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46388</v>
+        <v>46478</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>31305</v>
+        <v>789525</v>
       </c>
       <c r="I36" t="n">
-        <v>185.14</v>
+        <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>185.13</v>
+        <v>32.14</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>147194</v>
+        <v>79987</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I37" t="n">
-        <v>7.99</v>
+        <v>111.1</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
@@ -1855,39 +1855,39 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>148828</v>
+        <v>102636</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>4Q6489</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>792019</v>
+        <v>53333</v>
       </c>
       <c r="I38" t="n">
-        <v>93.70999999999999</v>
+        <v>11.39</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>11.39</v>
       </c>
     </row>
     <row r="39">
@@ -1897,35 +1897,35 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>153194</v>
+        <v>110370</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>0000293059</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I39" t="n">
-        <v>64.01000000000001</v>
+        <v>62.52</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="40">
@@ -1943,27 +1943,27 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>155970</v>
+        <v>142124</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I40" t="n">
-        <v>283.62</v>
+        <v>185.14</v>
       </c>
       <c r="J40" t="n">
-        <v>283.62</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="41">
@@ -1981,87 +1981,87 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>81973</v>
+        <v>147194</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>47252</v>
+        <v>33928</v>
       </c>
       <c r="I41" t="n">
-        <v>6.24</v>
+        <v>7.99</v>
       </c>
       <c r="J41" t="n">
-        <v>6.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>102393</v>
+        <v>148828</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4O3174</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46357</v>
+        <v>46508</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H42" t="n">
-        <v>53333</v>
+        <v>792019</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J42" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>142672</v>
+        <v>153194</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>0000293059</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
@@ -2071,39 +2071,39 @@
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>789429</v>
+        <v>789423</v>
       </c>
       <c r="I43" t="n">
-        <v>39.31</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="J43" t="n">
-        <v>39.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>142886</v>
+        <v>155970</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
@@ -2112,86 +2112,86 @@
         <v>789423</v>
       </c>
       <c r="I44" t="n">
-        <v>65.23999999999999</v>
+        <v>283.62</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>53</v>
+        <v>147</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>153194</v>
+        <v>81973</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I45" t="n">
-        <v>155.28</v>
+        <v>6.24</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>155919</v>
+        <v>102393</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I46" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
-        <v>158.77</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="47">
@@ -2209,27 +2209,27 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>159083</v>
+        <v>142672</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>794365</v>
+        <v>789429</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
       <c r="J47" t="n">
-        <v>88.59999999999999</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="48">
@@ -2239,149 +2239,149 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>55476</v>
+        <v>142886</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J48" t="n">
-        <v>56.83</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>66958</v>
+        <v>153194</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>789525</v>
+        <v>789423</v>
       </c>
       <c r="I49" t="n">
-        <v>59.39</v>
+        <v>155.28</v>
       </c>
       <c r="J49" t="n">
-        <v>59.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>92720</v>
+        <v>155919</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H50" t="n">
-        <v>37273</v>
+        <v>789423</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
       <c r="J50" t="n">
-        <v>6.88</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>100471</v>
+        <v>159083</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>4P2788</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H51" t="n">
-        <v>53333</v>
+        <v>794365</v>
       </c>
       <c r="I51" t="n">
-        <v>126.28</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>126.28</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="52">
@@ -2391,111 +2391,111 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>140760</v>
+        <v>55476</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>789423</v>
+        <v>30791</v>
       </c>
       <c r="I52" t="n">
-        <v>37.39</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>37.39</v>
+        <v>85.26000000000001</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>125</v>
+        <v>58</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>145507</v>
+        <v>66958</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46485</v>
+        <v>46478</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H53" t="n">
-        <v>47252</v>
+        <v>789525</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>59.39</v>
       </c>
       <c r="J53" t="n">
-        <v>26.34</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>160073</v>
+        <v>92720</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H54" t="n">
-        <v>795751</v>
+        <v>37273</v>
       </c>
       <c r="I54" t="n">
-        <v>74.92</v>
+        <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="55">
@@ -2513,87 +2513,87 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>44733</v>
+        <v>100471</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>46113</v>
+        <v>46419</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H55" t="n">
-        <v>790283</v>
+        <v>53333</v>
       </c>
       <c r="I55" t="n">
-        <v>27.55</v>
+        <v>126.28</v>
       </c>
       <c r="J55" t="n">
-        <v>27.55</v>
+        <v>126.28</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>49964</v>
+        <v>113662</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>OB1115</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H56" t="n">
-        <v>789228</v>
+        <v>31267</v>
       </c>
       <c r="I56" t="n">
-        <v>82.84999999999999</v>
+        <v>37.31</v>
       </c>
       <c r="J56" t="n">
-        <v>82.84999999999999</v>
+        <v>37.31</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>55204</v>
+        <v>140760</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
@@ -2603,73 +2603,73 @@
         <v>46259</v>
       </c>
       <c r="H57" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I57" t="n">
-        <v>43.92</v>
+        <v>37.39</v>
       </c>
       <c r="J57" t="n">
-        <v>43.92</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>84824</v>
+        <v>145507</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>46508</v>
+        <v>46485</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H58" t="n">
-        <v>789662</v>
+        <v>47252</v>
       </c>
       <c r="I58" t="n">
-        <v>27.31</v>
+        <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>0</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>125</v>
+        <v>38</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>88358</v>
+        <v>150514</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>4T3212</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
@@ -2679,48 +2679,48 @@
         <v>46259</v>
       </c>
       <c r="H59" t="n">
-        <v>793056</v>
+        <v>53333</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
+        <v>132.25</v>
       </c>
       <c r="J59" t="n">
-        <v>42.8</v>
+        <v>132.25</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>101583</v>
+        <v>160073</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>4V6234</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H60" t="n">
-        <v>53333</v>
+        <v>795751</v>
       </c>
       <c r="I60" t="n">
-        <v>125.05</v>
+        <v>74.92</v>
       </c>
       <c r="J60" t="n">
         <v>0</v>
@@ -2729,39 +2729,39 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>53</v>
+        <v>120</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>105546</v>
+        <v>44733</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>46419</v>
+        <v>46113</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H61" t="n">
-        <v>789423</v>
+        <v>790283</v>
       </c>
       <c r="I61" t="n">
-        <v>186.49</v>
+        <v>27.55</v>
       </c>
       <c r="J61" t="n">
-        <v>0</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="62">
@@ -2779,87 +2779,87 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>106348</v>
+        <v>49964</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>46478</v>
+        <v>46419</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H62" t="n">
-        <v>65455</v>
+        <v>789228</v>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J62" t="n">
-        <v>11.29</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>106364</v>
+        <v>55204</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H63" t="n">
-        <v>65455</v>
+        <v>30791</v>
       </c>
       <c r="I63" t="n">
-        <v>51.35</v>
+        <v>43.92</v>
       </c>
       <c r="J63" t="n">
-        <v>51.35</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>96</v>
+        <v>147</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>142645</v>
+        <v>84824</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
@@ -2869,35 +2869,35 @@
         <v>46259</v>
       </c>
       <c r="H64" t="n">
-        <v>789429</v>
+        <v>789662</v>
       </c>
       <c r="I64" t="n">
-        <v>81.64</v>
+        <v>27.31</v>
       </c>
       <c r="J64" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>146095</v>
+        <v>88358</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
@@ -2907,13 +2907,13 @@
         <v>46259</v>
       </c>
       <c r="H65" t="n">
-        <v>790283</v>
+        <v>793056</v>
       </c>
       <c r="I65" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>20.67</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="66">
@@ -2931,62 +2931,62 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>148816</v>
+        <v>101583</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>4V6234</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H66" t="n">
-        <v>33928</v>
+        <v>53333</v>
       </c>
       <c r="I66" t="n">
-        <v>10.43</v>
+        <v>125.05</v>
       </c>
       <c r="J66" t="n">
-        <v>10.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>148823</v>
+        <v>105546</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H67" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I67" t="n">
-        <v>53.82</v>
+        <v>186.49</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -3007,26 +3007,254 @@
         </is>
       </c>
       <c r="D68" t="n">
+        <v>106348</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>BR181245</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H68" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>11.29</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>125</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G69" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H69" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I69" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="J69" t="n">
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>96</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>SILAS SALVIANO PRATI</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>142645</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>25E17F</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H70" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I70" t="n">
+        <v>81.64</v>
+      </c>
+      <c r="J70" t="n">
+        <v>81.64</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>39</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G71" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H71" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I71" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J71" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>147</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G72" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H72" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I72" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J72" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>39</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G73" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H73" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I73" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>39</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
         <v>157761</v>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F68" s="2" t="n">
+      <c r="F74" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G68" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H68" t="n">
+      <c r="G74" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H74" t="n">
         <v>790808</v>
       </c>
-      <c r="I68" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" t="n">
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 16:45:03
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -943,77 +943,77 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>142466</v>
+        <v>140908</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>25I07B</t>
+          <t>3229-007-25</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H14" t="n">
-        <v>789429</v>
+        <v>30</v>
       </c>
       <c r="I14" t="n">
-        <v>39.97</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="J14" t="n">
-        <v>457.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>155114</v>
+        <v>142466</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0000267854</t>
+          <t>25I07B</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46327</v>
+        <v>46419</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H15" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I15" t="n">
-        <v>84.31</v>
+        <v>39.97</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>457.31</v>
       </c>
     </row>
     <row r="16">
@@ -1023,35 +1023,35 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>95052</v>
+        <v>155114</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>570950</t>
+          <t>0000267854</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46508</v>
+        <v>46327</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H16" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>84.31</v>
       </c>
       <c r="J16" t="n">
-        <v>312.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1069,100 +1069,100 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>98663</v>
+        <v>95052</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>4R6305</t>
+          <t>570950</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>37273</v>
+        <v>47252</v>
       </c>
       <c r="I17" t="n">
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>29.51</v>
+        <v>312.35</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>102024</v>
+        <v>98663</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4P0969</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46357</v>
+        <v>46447</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>53333</v>
+        <v>37273</v>
       </c>
       <c r="I18" t="n">
-        <v>18.67</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>0</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>110264</v>
+        <v>102024</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>B25B0673</t>
+          <t>4P0969</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I19" t="n">
-        <v>9.35</v>
+        <v>18.67</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1171,36 +1171,36 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>115223</v>
+        <v>110264</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>B25B0673</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I20" t="n">
-        <v>62.07</v>
+        <v>9.35</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1209,39 +1209,39 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
+        <v>62.07</v>
       </c>
       <c r="J21" t="n">
-        <v>346.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1251,57 +1251,57 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>39</v>
+        <v>80</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>153462</v>
+        <v>118036</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>30791</v>
+        <v>790808</v>
       </c>
       <c r="I22" t="n">
-        <v>1302.28</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>145</v>
+        <v>52</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>GVBA OL HERTZ ARTHUR DOS SANTOS</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>158962</v>
+        <v>153194</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1311,13 +1311,13 @@
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>793718</v>
+        <v>789423</v>
       </c>
       <c r="I23" t="n">
-        <v>196.61</v>
+        <v>26.34</v>
       </c>
       <c r="J23" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -1335,129 +1335,129 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>20206</v>
+        <v>153462</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PR1365</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>789228</v>
+        <v>30791</v>
       </c>
       <c r="I24" t="n">
-        <v>33.96</v>
+        <v>1302.28</v>
       </c>
       <c r="J24" t="n">
-        <v>33.96</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>38</v>
+        <v>145</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>64130</v>
+        <v>158962</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>45870</v>
+        <v>46508</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>30791</v>
+        <v>793718</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
+        <v>196.61</v>
       </c>
       <c r="J25" t="n">
-        <v>476.1</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>120901</v>
+        <v>20206</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>46327</v>
+        <v>46508</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>33057</v>
+        <v>789228</v>
       </c>
       <c r="I26" t="n">
-        <v>81.26000000000001</v>
+        <v>33.96</v>
       </c>
       <c r="J26" t="n">
-        <v>0</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>123315</v>
+        <v>64130</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>65651413</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>46419</v>
+        <v>45870</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>46259</v>
@@ -1469,143 +1469,143 @@
         <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>24.64</v>
+        <v>476.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>139865</v>
+        <v>120901</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>794365</v>
+        <v>33057</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J28" t="n">
-        <v>117.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>152839</v>
+        <v>123315</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>65651413</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>5582</v>
+        <v>30791</v>
       </c>
       <c r="I29" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>80.55</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>154122</v>
+        <v>139865</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>794919</v>
+        <v>794365</v>
       </c>
       <c r="I30" t="n">
-        <v>150.95</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>150.95</v>
+        <v>117.18</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>155008</v>
+        <v>152839</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -1615,13 +1615,13 @@
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>790283</v>
+        <v>5582</v>
       </c>
       <c r="I31" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
       <c r="J31" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="32">
@@ -1639,129 +1639,129 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>155969</v>
+        <v>154122</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>789423</v>
+        <v>794919</v>
       </c>
       <c r="I32" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
       <c r="J32" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>55476</v>
+        <v>155008</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>30791</v>
+        <v>790283</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
+        <v>18.72</v>
       </c>
       <c r="J33" t="n">
-        <v>56.86</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>55476</v>
+        <v>155969</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>510.49</v>
       </c>
       <c r="J34" t="n">
-        <v>113.71</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>64130</v>
+        <v>55476</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>45870</v>
+        <v>46478</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
@@ -1770,10 +1770,10 @@
         <v>30791</v>
       </c>
       <c r="I35" t="n">
-        <v>59.5</v>
+        <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>59.5</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="36">
@@ -1791,11 +1791,11 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>66958</v>
+        <v>55476</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
@@ -1805,115 +1805,115 @@
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>789525</v>
+        <v>30791</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>32.14</v>
+        <v>113.71</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>79987</v>
+        <v>64130</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>B25B1713</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46447</v>
+        <v>45870</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I37" t="n">
-        <v>111.1</v>
+        <v>59.5</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>102636</v>
+        <v>66958</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>4Q6489</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>53333</v>
+        <v>789525</v>
       </c>
       <c r="I38" t="n">
-        <v>11.39</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>11.39</v>
+        <v>32.14</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>110370</v>
+        <v>79987</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
@@ -1922,48 +1922,48 @@
         <v>47252</v>
       </c>
       <c r="I39" t="n">
-        <v>62.52</v>
+        <v>111.1</v>
       </c>
       <c r="J39" t="n">
-        <v>62.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>142124</v>
+        <v>102636</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>4Q6489</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>31305</v>
+        <v>53333</v>
       </c>
       <c r="I40" t="n">
-        <v>185.14</v>
+        <v>11.39</v>
       </c>
       <c r="J40" t="n">
-        <v>185.13</v>
+        <v>11.39</v>
       </c>
     </row>
     <row r="41">
@@ -1981,11 +1981,11 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>147194</v>
+        <v>110370</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -1995,51 +1995,51 @@
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I41" t="n">
-        <v>7.99</v>
+        <v>62.52</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>148828</v>
+        <v>142124</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H42" t="n">
-        <v>792019</v>
+        <v>31305</v>
       </c>
       <c r="I42" t="n">
-        <v>93.70999999999999</v>
+        <v>185.14</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="43">
@@ -2049,32 +2049,32 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>153194</v>
+        <v>147194</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0000293059</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I43" t="n">
-        <v>64.01000000000001</v>
+        <v>7.99</v>
       </c>
       <c r="J43" t="n">
         <v>0</v>
@@ -2083,23 +2083,23 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>155970</v>
+        <v>148828</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
@@ -2109,13 +2109,13 @@
         <v>46259</v>
       </c>
       <c r="H44" t="n">
-        <v>789423</v>
+        <v>792019</v>
       </c>
       <c r="I44" t="n">
-        <v>283.62</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J44" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -2125,111 +2125,111 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>81973</v>
+        <v>153194</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>0000293059</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I45" t="n">
-        <v>6.24</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="J45" t="n">
-        <v>6.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>102393</v>
+        <v>155970</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4O3174</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46357</v>
+        <v>46508</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>53333</v>
+        <v>789423</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>283.62</v>
       </c>
       <c r="J46" t="n">
-        <v>2.02</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>142672</v>
+        <v>81973</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I47" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
       <c r="J47" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="48">
@@ -2239,57 +2239,57 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>142886</v>
+        <v>102393</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I48" t="n">
-        <v>65.23999999999999</v>
+        <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>153194</v>
+        <v>142672</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -2299,35 +2299,35 @@
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I49" t="n">
-        <v>155.28</v>
+        <v>39.31</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>155919</v>
+        <v>142886</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
@@ -2340,124 +2340,124 @@
         <v>789423</v>
       </c>
       <c r="I50" t="n">
-        <v>158.77</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="J50" t="n">
-        <v>158.77</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>159083</v>
+        <v>153194</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H51" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>155.28</v>
       </c>
       <c r="J51" t="n">
-        <v>88.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>55476</v>
+        <v>155919</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
       <c r="J52" t="n">
-        <v>85.26000000000001</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>58</v>
+        <v>125</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>66958</v>
+        <v>159083</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H53" t="n">
-        <v>789525</v>
+        <v>794365</v>
       </c>
       <c r="I53" t="n">
-        <v>59.39</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>59.39</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="54">
@@ -2467,35 +2467,35 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>92720</v>
+        <v>55476</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H54" t="n">
-        <v>37273</v>
+        <v>30791</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>6.88</v>
+        <v>85.26000000000001</v>
       </c>
     </row>
     <row r="55">
@@ -2505,225 +2505,225 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>100471</v>
+        <v>66958</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>4P2788</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H55" t="n">
-        <v>53333</v>
+        <v>789525</v>
       </c>
       <c r="I55" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
       <c r="J55" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>113662</v>
+        <v>92720</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>OB1115</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H56" t="n">
-        <v>31267</v>
+        <v>37273</v>
       </c>
       <c r="I56" t="n">
-        <v>37.31</v>
+        <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>37.31</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>140760</v>
+        <v>100471</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H57" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I57" t="n">
-        <v>37.39</v>
+        <v>126.28</v>
       </c>
       <c r="J57" t="n">
-        <v>37.39</v>
+        <v>126.28</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>125</v>
+        <v>38</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>145507</v>
+        <v>113662</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>OB1115</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>46485</v>
+        <v>46478</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H58" t="n">
-        <v>47252</v>
+        <v>31267</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>37.31</v>
       </c>
       <c r="J58" t="n">
-        <v>26.34</v>
+        <v>37.31</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>38</v>
+        <v>111</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>150514</v>
+        <v>140760</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>4T3212</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H59" t="n">
-        <v>53333</v>
+        <v>789423</v>
       </c>
       <c r="I59" t="n">
-        <v>132.25</v>
+        <v>37.39</v>
       </c>
       <c r="J59" t="n">
-        <v>132.25</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>160073</v>
+        <v>145507</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>46447</v>
+        <v>46485</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H60" t="n">
-        <v>795751</v>
+        <v>47252</v>
       </c>
       <c r="I60" t="n">
-        <v>74.92</v>
+        <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>0</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="61">
@@ -2733,57 +2733,57 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>44733</v>
+        <v>150514</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>4T3212</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>46113</v>
+        <v>46508</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H61" t="n">
-        <v>790283</v>
+        <v>53333</v>
       </c>
       <c r="I61" t="n">
-        <v>27.55</v>
+        <v>132.25</v>
       </c>
       <c r="J61" t="n">
-        <v>27.55</v>
+        <v>132.25</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>49964</v>
+        <v>157673</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>0525</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
@@ -2793,13 +2793,13 @@
         <v>46259</v>
       </c>
       <c r="H62" t="n">
-        <v>789228</v>
+        <v>47252</v>
       </c>
       <c r="I62" t="n">
-        <v>82.84999999999999</v>
+        <v>13.09</v>
       </c>
       <c r="J62" t="n">
-        <v>82.84999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63">
@@ -2817,11 +2817,11 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>55204</v>
+        <v>160073</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
@@ -2831,162 +2831,162 @@
         <v>46259</v>
       </c>
       <c r="H63" t="n">
-        <v>30791</v>
+        <v>795751</v>
       </c>
       <c r="I63" t="n">
-        <v>43.92</v>
+        <v>74.92</v>
       </c>
       <c r="J63" t="n">
-        <v>43.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>84824</v>
+        <v>44733</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>46508</v>
+        <v>46113</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H64" t="n">
-        <v>789662</v>
+        <v>790283</v>
       </c>
       <c r="I64" t="n">
-        <v>27.31</v>
+        <v>27.55</v>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>88358</v>
+        <v>49964</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H65" t="n">
-        <v>793056</v>
+        <v>789228</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J65" t="n">
-        <v>42.8</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>101583</v>
+        <v>55204</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>4V6234</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H66" t="n">
-        <v>53333</v>
+        <v>30791</v>
       </c>
       <c r="I66" t="n">
-        <v>125.05</v>
+        <v>43.92</v>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>53</v>
+        <v>147</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>105546</v>
+        <v>84824</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H67" t="n">
-        <v>789423</v>
+        <v>789662</v>
       </c>
       <c r="I67" t="n">
-        <v>186.49</v>
+        <v>27.31</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -2995,61 +2995,61 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>106348</v>
+        <v>88358</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H68" t="n">
-        <v>65455</v>
+        <v>793056</v>
       </c>
       <c r="I68" t="n">
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>11.29</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>106364</v>
+        <v>101583</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>4V6234</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
@@ -3059,51 +3059,51 @@
         <v>46259</v>
       </c>
       <c r="H69" t="n">
-        <v>65455</v>
+        <v>53333</v>
       </c>
       <c r="I69" t="n">
-        <v>51.35</v>
+        <v>125.05</v>
       </c>
       <c r="J69" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>142645</v>
+        <v>105546</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G70" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H70" t="n">
-        <v>789429</v>
+        <v>789423</v>
       </c>
       <c r="I70" t="n">
-        <v>81.64</v>
+        <v>186.49</v>
       </c>
       <c r="J70" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -3121,103 +3121,103 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>146095</v>
+        <v>106348</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H71" t="n">
-        <v>790283</v>
+        <v>65455</v>
       </c>
       <c r="I71" t="n">
-        <v>8.15</v>
+        <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>20.67</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>148816</v>
+        <v>106364</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H72" t="n">
-        <v>33928</v>
+        <v>65455</v>
       </c>
       <c r="I72" t="n">
-        <v>10.43</v>
+        <v>51.35</v>
       </c>
       <c r="J72" t="n">
-        <v>10.43</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>39</v>
+        <v>96</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>148823</v>
+        <v>142645</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>25E17F</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H73" t="n">
-        <v>33928</v>
+        <v>789429</v>
       </c>
       <c r="I73" t="n">
-        <v>53.82</v>
+        <v>81.64</v>
       </c>
       <c r="J73" t="n">
-        <v>0</v>
+        <v>81.64</v>
       </c>
     </row>
     <row r="74">
@@ -3235,26 +3235,140 @@
         </is>
       </c>
       <c r="D74" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G74" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H74" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I74" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J74" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>147</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G75" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H75" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I75" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J75" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>39</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H76" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I76" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>39</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
         <v>157761</v>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F74" s="2" t="n">
+      <c r="F77" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G74" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H74" t="n">
+      <c r="G77" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H77" t="n">
         <v>790808</v>
       </c>
-      <c r="I74" t="n">
-        <v>0</v>
-      </c>
-      <c r="J74" t="n">
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 17:00:03
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -829,65 +829,65 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>79375</v>
+        <v>67369</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>B25H1773</t>
+          <t>2522571</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H11" t="n">
-        <v>47252</v>
+        <v>29</v>
       </c>
       <c r="I11" t="n">
-        <v>150.28</v>
+        <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>0</v>
+        <v>103.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>79995</v>
+        <v>79375</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>B25B2383</t>
+          <t>B25H1773</t>
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>46259</v>
@@ -896,7 +896,7 @@
         <v>47252</v>
       </c>
       <c r="I12" t="n">
-        <v>144.41</v>
+        <v>150.28</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -905,153 +905,153 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>139865</v>
+        <v>79995</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>B25B2383</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H13" t="n">
-        <v>794365</v>
+        <v>47252</v>
       </c>
       <c r="I13" t="n">
-        <v>25.42</v>
+        <v>144.41</v>
       </c>
       <c r="J13" t="n">
-        <v>25.42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>38</v>
+        <v>145</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>140908</v>
+        <v>139865</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>3229-007-25</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H14" t="n">
-        <v>30</v>
+        <v>794365</v>
       </c>
       <c r="I14" t="n">
-        <v>97.90000000000001</v>
+        <v>25.42</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>25.42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>142466</v>
+        <v>140908</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>25I07B</t>
+          <t>3229-007-25</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H15" t="n">
-        <v>789429</v>
+        <v>30</v>
       </c>
       <c r="I15" t="n">
-        <v>39.97</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="J15" t="n">
-        <v>457.31</v>
+        <v>97.90000000000001</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>111</v>
+        <v>39</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>155114</v>
+        <v>142466</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0000267854</t>
+          <t>25I07B</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>46327</v>
+        <v>46419</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H16" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I16" t="n">
-        <v>84.31</v>
+        <v>39.97</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>457.31</v>
       </c>
     </row>
     <row r="17">
@@ -1061,35 +1061,35 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>95052</v>
+        <v>155114</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>570950</t>
+          <t>0000267854</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
-        <v>46508</v>
+        <v>46327</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H17" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>84.33</v>
       </c>
       <c r="J17" t="n">
-        <v>312.35</v>
+        <v>84.33</v>
       </c>
     </row>
     <row r="18">
@@ -1107,100 +1107,100 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>98663</v>
+        <v>95052</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>4R6305</t>
+          <t>570950</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>37273</v>
+        <v>47252</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>29.51</v>
+        <v>312.35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>102024</v>
+        <v>98663</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4P0969</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46357</v>
+        <v>46447</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>53333</v>
+        <v>37273</v>
       </c>
       <c r="I19" t="n">
-        <v>18.67</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>0</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>110264</v>
+        <v>102024</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>B25B0673</t>
+          <t>4P0969</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I20" t="n">
-        <v>9.35</v>
+        <v>18.67</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1209,36 +1209,36 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>115223</v>
+        <v>110264</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>B25B0673</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I21" t="n">
-        <v>62.07</v>
+        <v>9.35</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1247,61 +1247,61 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
+        <v>62.08</v>
       </c>
       <c r="J22" t="n">
-        <v>346.2</v>
+        <v>62.08</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ ARTHUR DOS SANTOS</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>153194</v>
+        <v>118036</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1311,48 +1311,48 @@
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>789423</v>
+        <v>790808</v>
       </c>
       <c r="I23" t="n">
-        <v>26.34</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ ARTHUR DOS SANTOS</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>153462</v>
+        <v>153194</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I24" t="n">
-        <v>1302.28</v>
+        <v>26.34</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
@@ -1361,61 +1361,61 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>158962</v>
+        <v>153462</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="I25" t="n">
-        <v>196.61</v>
+        <v>1302.28</v>
       </c>
       <c r="J25" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>20206</v>
+        <v>158962</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PR1365</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -1425,263 +1425,263 @@
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="I26" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
       <c r="J26" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>64130</v>
+        <v>20206</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
-        <v>45870</v>
+        <v>46508</v>
       </c>
       <c r="G27" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>33.96</v>
       </c>
       <c r="J27" t="n">
-        <v>476.1</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>120901</v>
+        <v>64130</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>46327</v>
+        <v>45870</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>33057</v>
+        <v>30791</v>
       </c>
       <c r="I28" t="n">
-        <v>81.26000000000001</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>0</v>
+        <v>476.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>106</v>
+        <v>38</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>123315</v>
+        <v>66958</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>65651413</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>30791</v>
+        <v>789525</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>24.64</v>
+        <v>30.23</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>139865</v>
+        <v>120901</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>794365</v>
+        <v>33057</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J30" t="n">
-        <v>117.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>152839</v>
+        <v>123315</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>65651413</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>5582</v>
+        <v>30791</v>
       </c>
       <c r="I31" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>80.55</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>154122</v>
+        <v>139865</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>794919</v>
+        <v>794365</v>
       </c>
       <c r="I32" t="n">
-        <v>150.95</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>150.95</v>
+        <v>117.18</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>155008</v>
+        <v>152839</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
@@ -1691,13 +1691,13 @@
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>790283</v>
+        <v>5582</v>
       </c>
       <c r="I33" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
       <c r="J33" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="34">
@@ -1715,141 +1715,141 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>155969</v>
+        <v>154122</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>789423</v>
+        <v>794919</v>
       </c>
       <c r="I34" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
       <c r="J34" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>55476</v>
+        <v>155008</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>30791</v>
+        <v>790283</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>18.72</v>
       </c>
       <c r="J35" t="n">
-        <v>56.86</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>55476</v>
+        <v>155969</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>510.49</v>
       </c>
       <c r="J36" t="n">
-        <v>113.71</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>120</v>
+        <v>147</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>64130</v>
+        <v>16217</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>5I9866</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>45870</v>
+        <v>46419</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>30791</v>
+        <v>33286</v>
       </c>
       <c r="I37" t="n">
-        <v>59.5</v>
+        <v>12.98</v>
       </c>
       <c r="J37" t="n">
-        <v>59.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -1859,19 +1859,19 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>66958</v>
+        <v>55476</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
@@ -1881,51 +1881,51 @@
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>789525</v>
+        <v>30791</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>32.14</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>79987</v>
+        <v>55476</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>B25B1713</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I39" t="n">
-        <v>111.1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>113.71</v>
       </c>
     </row>
     <row r="40">
@@ -1935,73 +1935,73 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>102636</v>
+        <v>64130</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>4Q6489</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>46419</v>
+        <v>45870</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H40" t="n">
-        <v>53333</v>
+        <v>30791</v>
       </c>
       <c r="I40" t="n">
-        <v>11.39</v>
+        <v>59.5</v>
       </c>
       <c r="J40" t="n">
-        <v>11.39</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>110370</v>
+        <v>66958</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
-        <v>46388</v>
+        <v>46478</v>
       </c>
       <c r="G41" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>47252</v>
+        <v>789525</v>
       </c>
       <c r="I41" t="n">
-        <v>62.52</v>
+        <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>62.52</v>
+        <v>32.14</v>
       </c>
     </row>
     <row r="42">
@@ -2019,65 +2019,65 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>142124</v>
+        <v>79987</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H42" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I42" t="n">
-        <v>185.14</v>
+        <v>111.1</v>
       </c>
       <c r="J42" t="n">
-        <v>185.13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>147194</v>
+        <v>102636</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>4Q6489</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>33928</v>
+        <v>53333</v>
       </c>
       <c r="I43" t="n">
-        <v>7.99</v>
+        <v>11.39</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>11.39</v>
       </c>
     </row>
     <row r="44">
@@ -2095,103 +2095,103 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>148828</v>
+        <v>110370</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H44" t="n">
-        <v>792019</v>
+        <v>47252</v>
       </c>
       <c r="I44" t="n">
-        <v>93.70999999999999</v>
+        <v>62.52</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>142</v>
+        <v>39</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>153194</v>
+        <v>142124</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>0000293059</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>789423</v>
+        <v>31305</v>
       </c>
       <c r="I45" t="n">
-        <v>64.01000000000001</v>
+        <v>185.14</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>155970</v>
+        <v>147194</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I46" t="n">
-        <v>283.62</v>
+        <v>7.99</v>
       </c>
       <c r="J46" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -2209,87 +2209,87 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>81973</v>
+        <v>148828</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>47252</v>
+        <v>792019</v>
       </c>
       <c r="I47" t="n">
-        <v>6.24</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J47" t="n">
-        <v>6.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>102393</v>
+        <v>153194</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>4O3174</t>
+          <t>0000293059</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46357</v>
+        <v>46508</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>53333</v>
+        <v>789423</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="J48" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>142672</v>
+        <v>155970</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -2299,127 +2299,127 @@
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>789429</v>
+        <v>789423</v>
       </c>
       <c r="I49" t="n">
-        <v>39.31</v>
+        <v>283.62</v>
       </c>
       <c r="J49" t="n">
-        <v>39.31</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>142886</v>
+        <v>81973</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H50" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I50" t="n">
-        <v>65.23999999999999</v>
+        <v>6.24</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>53</v>
+        <v>106</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>153194</v>
+        <v>102393</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46508</v>
+        <v>46357</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H51" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I51" t="n">
-        <v>155.28</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>155919</v>
+        <v>142672</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I52" t="n">
-        <v>158.77</v>
+        <v>39.31</v>
       </c>
       <c r="J52" t="n">
-        <v>158.77</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="53">
@@ -2429,111 +2429,111 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>159083</v>
+        <v>142886</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46447</v>
+        <v>46388</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H53" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>65.25</v>
       </c>
       <c r="J53" t="n">
-        <v>88.59999999999999</v>
+        <v>32.63</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>106</v>
+        <v>53</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>55476</v>
+        <v>153194</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H54" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
+        <v>155.28</v>
       </c>
       <c r="J54" t="n">
-        <v>85.26000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>66958</v>
+        <v>155919</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>46478</v>
+        <v>46388</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H55" t="n">
-        <v>789525</v>
+        <v>789423</v>
       </c>
       <c r="I55" t="n">
-        <v>59.39</v>
+        <v>158.77</v>
       </c>
       <c r="J55" t="n">
-        <v>59.39</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="56">
@@ -2551,27 +2551,27 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>92720</v>
+        <v>159083</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H56" t="n">
-        <v>37273</v>
+        <v>794365</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
       </c>
       <c r="J56" t="n">
-        <v>6.88</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -2589,49 +2589,49 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>100471</v>
+        <v>17310</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>4P2788</t>
+          <t>B25E1014</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H57" t="n">
-        <v>53333</v>
+        <v>47252</v>
       </c>
       <c r="I57" t="n">
-        <v>126.28</v>
+        <v>49.4</v>
       </c>
       <c r="J57" t="n">
-        <v>126.28</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>113662</v>
+        <v>55476</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>OB1115</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
@@ -2641,51 +2641,51 @@
         <v>46259</v>
       </c>
       <c r="H58" t="n">
-        <v>31267</v>
+        <v>30791</v>
       </c>
       <c r="I58" t="n">
-        <v>37.31</v>
+        <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>37.31</v>
+        <v>85.26000000000001</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>140760</v>
+        <v>66958</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H59" t="n">
-        <v>789423</v>
+        <v>789525</v>
       </c>
       <c r="I59" t="n">
-        <v>37.39</v>
+        <v>59.39</v>
       </c>
       <c r="J59" t="n">
-        <v>37.39</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="60">
@@ -2703,27 +2703,27 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>145507</v>
+        <v>92720</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>46485</v>
+        <v>46508</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H60" t="n">
-        <v>47252</v>
+        <v>37273</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>26.34</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="61">
@@ -2733,23 +2733,23 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>38</v>
+        <v>120</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>150514</v>
+        <v>100471</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>4T3212</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>46259</v>
@@ -2758,70 +2758,70 @@
         <v>53333</v>
       </c>
       <c r="I61" t="n">
-        <v>132.25</v>
+        <v>126.28</v>
       </c>
       <c r="J61" t="n">
-        <v>132.25</v>
+        <v>126.28</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>125</v>
+        <v>38</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>157673</v>
+        <v>113662</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>0525</t>
+          <t>OB1115</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H62" t="n">
-        <v>47252</v>
+        <v>31267</v>
       </c>
       <c r="I62" t="n">
-        <v>13.09</v>
+        <v>100.89</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>37.31</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>160073</v>
+        <v>140760</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
@@ -2831,162 +2831,162 @@
         <v>46259</v>
       </c>
       <c r="H63" t="n">
-        <v>795751</v>
+        <v>789423</v>
       </c>
       <c r="I63" t="n">
-        <v>74.92</v>
+        <v>37.39</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>44733</v>
+        <v>145507</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>46113</v>
+        <v>46485</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H64" t="n">
-        <v>790283</v>
+        <v>47252</v>
       </c>
       <c r="I64" t="n">
-        <v>27.55</v>
+        <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>27.55</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>39</v>
+        <v>142</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>49964</v>
+        <v>145709</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>0000277236</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H65" t="n">
-        <v>789228</v>
+        <v>789423</v>
       </c>
       <c r="I65" t="n">
-        <v>82.84999999999999</v>
+        <v>49.42</v>
       </c>
       <c r="J65" t="n">
-        <v>82.84999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>55204</v>
+        <v>150514</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>4T3212</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H66" t="n">
-        <v>30791</v>
+        <v>53333</v>
       </c>
       <c r="I66" t="n">
-        <v>43.92</v>
+        <v>132.25</v>
       </c>
       <c r="J66" t="n">
-        <v>43.92</v>
+        <v>132.25</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>84824</v>
+        <v>157673</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>0525</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H67" t="n">
-        <v>789662</v>
+        <v>47252</v>
       </c>
       <c r="I67" t="n">
-        <v>27.31</v>
+        <v>13.09</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -2995,99 +2995,99 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>88358</v>
+        <v>160073</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H68" t="n">
-        <v>793056</v>
+        <v>795751</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
+        <v>74.92</v>
       </c>
       <c r="J68" t="n">
-        <v>42.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>147</v>
+        <v>120</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>101583</v>
+        <v>44733</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>4V6234</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>46508</v>
+        <v>46113</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H69" t="n">
-        <v>53333</v>
+        <v>790283</v>
       </c>
       <c r="I69" t="n">
-        <v>125.05</v>
+        <v>27.55</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>105546</v>
+        <v>49964</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
@@ -3097,13 +3097,13 @@
         <v>46259</v>
       </c>
       <c r="H70" t="n">
-        <v>789423</v>
+        <v>789228</v>
       </c>
       <c r="I70" t="n">
-        <v>186.49</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="71">
@@ -3121,49 +3121,49 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>106348</v>
+        <v>55204</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H71" t="n">
-        <v>65455</v>
+        <v>30791</v>
       </c>
       <c r="I71" t="n">
-        <v>0</v>
+        <v>43.92</v>
       </c>
       <c r="J71" t="n">
-        <v>11.29</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>106364</v>
+        <v>84824</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
@@ -3173,35 +3173,35 @@
         <v>46259</v>
       </c>
       <c r="H72" t="n">
-        <v>65455</v>
+        <v>789662</v>
       </c>
       <c r="I72" t="n">
-        <v>51.35</v>
+        <v>27.31</v>
       </c>
       <c r="J72" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>142645</v>
+        <v>88358</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
@@ -3211,35 +3211,35 @@
         <v>46259</v>
       </c>
       <c r="H73" t="n">
-        <v>789429</v>
+        <v>793056</v>
       </c>
       <c r="I73" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
       <c r="J73" t="n">
-        <v>81.64</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>146095</v>
+        <v>101583</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>4V6234</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
@@ -3249,51 +3249,51 @@
         <v>46259</v>
       </c>
       <c r="H74" t="n">
-        <v>790283</v>
+        <v>53333</v>
       </c>
       <c r="I74" t="n">
-        <v>8.15</v>
+        <v>125.05</v>
       </c>
       <c r="J74" t="n">
-        <v>20.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>147</v>
+        <v>53</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>148816</v>
+        <v>105546</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>46478</v>
+        <v>46419</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H75" t="n">
-        <v>33928</v>
+        <v>789423</v>
       </c>
       <c r="I75" t="n">
-        <v>10.43</v>
+        <v>186.49</v>
       </c>
       <c r="J75" t="n">
-        <v>10.43</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
@@ -3311,64 +3311,254 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>148823</v>
+        <v>106348</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H76" t="n">
-        <v>33928</v>
+        <v>65455</v>
       </c>
       <c r="I76" t="n">
-        <v>53.82</v>
+        <v>0</v>
       </c>
       <c r="J76" t="n">
-        <v>0</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>125</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>FERNANDO NOBRE MARTINS</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>106364</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>BR183284</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H77" t="n">
+        <v>65455</v>
+      </c>
+      <c r="I77" t="n">
+        <v>51.35</v>
+      </c>
+      <c r="J77" t="n">
+        <v>51.35</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>96</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>SILAS SALVIANO PRATI</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>142645</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>25E17F</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G78" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H78" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I78" t="n">
+        <v>81.64</v>
+      </c>
+      <c r="J78" t="n">
+        <v>81.64</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t>PI</t>
         </is>
       </c>
-      <c r="B77" t="n">
+      <c r="B79" t="n">
         <v>39</v>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D79" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G79" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H79" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I79" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J79" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>147</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G80" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H80" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I80" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J80" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>39</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G81" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H81" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I81" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>39</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
         <v>157761</v>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F77" s="2" t="n">
+      <c r="F82" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G77" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H77" t="n">
+      <c r="G82" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H82" t="n">
         <v>790808</v>
       </c>
-      <c r="I77" t="n">
-        <v>0</v>
-      </c>
-      <c r="J77" t="n">
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 17:15:03
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J82"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1095,23 +1095,23 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>125</v>
+        <v>26</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>95052</v>
+        <v>57088</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>570950</t>
+          <t>15172872</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -1121,13 +1121,13 @@
         <v>46259</v>
       </c>
       <c r="H18" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>20.04</v>
       </c>
       <c r="J18" t="n">
-        <v>312.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1145,100 +1145,100 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>98663</v>
+        <v>95052</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4R6305</t>
+          <t>570950</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H19" t="n">
-        <v>37273</v>
+        <v>47252</v>
       </c>
       <c r="I19" t="n">
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>29.51</v>
+        <v>312.35</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>102024</v>
+        <v>98663</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>4P0969</t>
+          <t>4R6305</t>
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>46357</v>
+        <v>46447</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H20" t="n">
-        <v>53333</v>
+        <v>37273</v>
       </c>
       <c r="I20" t="n">
-        <v>18.67</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>0</v>
+        <v>29.51</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>26</v>
+        <v>147</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>110264</v>
+        <v>102024</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>B25B0673</t>
+          <t>4P0969</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>46447</v>
+        <v>46357</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H21" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I21" t="n">
-        <v>9.35</v>
+        <v>18.67</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
@@ -1247,99 +1247,99 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t xml:space="preserve">SILAS SALVIANO DE SOUZA </t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>115223</v>
+        <v>110264</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0000275143</t>
+          <t>B25B0673</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H22" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I22" t="n">
-        <v>62.08</v>
+        <v>9.35</v>
       </c>
       <c r="J22" t="n">
-        <v>62.08</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>80</v>
+        <v>111</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GERUSIA MARIA DA SILVA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>118036</v>
+        <v>115223</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>4T9475</t>
+          <t>0000275143</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G23" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H23" t="n">
-        <v>790808</v>
+        <v>789423</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>62.08</v>
       </c>
       <c r="J23" t="n">
-        <v>346.2</v>
+        <v>62.08</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>52</v>
+        <v>80</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ ARTHUR DOS SANTOS</t>
+          <t>GERUSIA MARIA DA SILVA</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>153194</v>
+        <v>118036</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>4T9475</t>
         </is>
       </c>
       <c r="F24" s="2" t="n">
@@ -1349,48 +1349,48 @@
         <v>46259</v>
       </c>
       <c r="H24" t="n">
-        <v>789423</v>
+        <v>790808</v>
       </c>
       <c r="I24" t="n">
-        <v>26.34</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>346.2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ ARTHUR DOS SANTOS</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>153462</v>
+        <v>153194</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>68340022</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H25" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I25" t="n">
-        <v>1302.28</v>
+        <v>26.34</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1399,61 +1399,61 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>158962</v>
+        <v>153462</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>41103077</t>
+          <t>68340022</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H26" t="n">
-        <v>793718</v>
+        <v>30791</v>
       </c>
       <c r="I26" t="n">
-        <v>196.61</v>
+        <v>1302.28</v>
       </c>
       <c r="J26" t="n">
-        <v>196.61</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>20206</v>
+        <v>158962</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PR1365</t>
+          <t>41103077</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -1463,51 +1463,51 @@
         <v>46259</v>
       </c>
       <c r="H27" t="n">
-        <v>789228</v>
+        <v>793718</v>
       </c>
       <c r="I27" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
       <c r="J27" t="n">
-        <v>33.96</v>
+        <v>196.61</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>64130</v>
+        <v>20206</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>PR1365</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
-        <v>45870</v>
+        <v>46508</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H28" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
+        <v>33.96</v>
       </c>
       <c r="J28" t="n">
-        <v>476.1</v>
+        <v>33.96</v>
       </c>
     </row>
     <row r="29">
@@ -1525,239 +1525,239 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>66958</v>
+        <v>64130</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F29" s="2" t="n">
-        <v>46478</v>
+        <v>45870</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H29" t="n">
-        <v>789525</v>
+        <v>30791</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>30.23</v>
+        <v>476.1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>120901</v>
+        <v>66958</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0029956</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
-        <v>46327</v>
+        <v>46478</v>
       </c>
       <c r="G30" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H30" t="n">
-        <v>33057</v>
+        <v>789525</v>
       </c>
       <c r="I30" t="n">
-        <v>81.26000000000001</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>30.23</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>123315</v>
+        <v>82538</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>65651413</t>
+          <t>B25B2279</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H31" t="n">
-        <v>30791</v>
+        <v>47252</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
+        <v>71.88</v>
       </c>
       <c r="J31" t="n">
-        <v>24.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>139865</v>
+        <v>120901</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2500455</t>
+          <t>0029956</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
-        <v>46419</v>
+        <v>46327</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H32" t="n">
-        <v>794365</v>
+        <v>33057</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>81.26000000000001</v>
       </c>
       <c r="J32" t="n">
-        <v>117.18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>152839</v>
+        <v>123315</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>4O9571</t>
+          <t>65651413</t>
         </is>
       </c>
       <c r="F33" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H33" t="n">
-        <v>5582</v>
+        <v>30791</v>
       </c>
       <c r="I33" t="n">
-        <v>80.55</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>80.55</v>
+        <v>24.64</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>39</v>
+        <v>106</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>154122</v>
+        <v>139865</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>4Q0092</t>
+          <t>2500455</t>
         </is>
       </c>
       <c r="F34" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G34" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H34" t="n">
-        <v>794919</v>
+        <v>794365</v>
       </c>
       <c r="I34" t="n">
-        <v>150.95</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>150.95</v>
+        <v>117.18</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>155008</v>
+        <v>152839</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>255239</t>
+          <t>4O9571</t>
         </is>
       </c>
       <c r="F35" s="2" t="n">
@@ -1767,13 +1767,13 @@
         <v>46259</v>
       </c>
       <c r="H35" t="n">
-        <v>790283</v>
+        <v>5582</v>
       </c>
       <c r="I35" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
       <c r="J35" t="n">
-        <v>18.72</v>
+        <v>80.55</v>
       </c>
     </row>
     <row r="36">
@@ -1791,27 +1791,27 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>155969</v>
+        <v>154122</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>KN.040440</t>
+          <t>4Q0092</t>
         </is>
       </c>
       <c r="F36" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H36" t="n">
-        <v>789423</v>
+        <v>794919</v>
       </c>
       <c r="I36" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
       <c r="J36" t="n">
-        <v>510.49</v>
+        <v>150.95</v>
       </c>
     </row>
     <row r="37">
@@ -1829,129 +1829,129 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>16217</v>
+        <v>155008</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>5I9866</t>
+          <t>255239</t>
         </is>
       </c>
       <c r="F37" s="2" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H37" t="n">
-        <v>33286</v>
+        <v>790283</v>
       </c>
       <c r="I37" t="n">
-        <v>12.98</v>
+        <v>18.72</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>18.72</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>145</v>
+        <v>39</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>55476</v>
+        <v>155969</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>KN.040440</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H38" t="n">
-        <v>30791</v>
+        <v>789423</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
+        <v>510.49</v>
       </c>
       <c r="J38" t="n">
-        <v>56.86</v>
+        <v>510.49</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>55476</v>
+        <v>16217</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>5I9866</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
-        <v>46478</v>
+        <v>46419</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H39" t="n">
-        <v>30791</v>
+        <v>33286</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
+        <v>12.98</v>
       </c>
       <c r="J39" t="n">
-        <v>113.71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>120</v>
+        <v>145</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>64130</v>
+        <v>55476</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>45870</v>
+        <v>46478</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>46259</v>
@@ -1960,10 +1960,10 @@
         <v>30791</v>
       </c>
       <c r="I40" t="n">
-        <v>59.5</v>
+        <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>59.5</v>
+        <v>56.86</v>
       </c>
     </row>
     <row r="41">
@@ -1981,11 +1981,11 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>66958</v>
+        <v>55476</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F41" s="2" t="n">
@@ -1995,115 +1995,115 @@
         <v>46259</v>
       </c>
       <c r="H41" t="n">
-        <v>789525</v>
+        <v>30791</v>
       </c>
       <c r="I41" t="n">
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>32.14</v>
+        <v>113.71</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>79987</v>
+        <v>64130</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>B25B1713</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>46447</v>
+        <v>45870</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H42" t="n">
-        <v>47252</v>
+        <v>30791</v>
       </c>
       <c r="I42" t="n">
-        <v>111.1</v>
+        <v>59.5</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>102636</v>
+        <v>66958</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>4Q6489</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>53333</v>
+        <v>789525</v>
       </c>
       <c r="I43" t="n">
-        <v>11.39</v>
+        <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>11.39</v>
+        <v>32.14</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>110370</v>
+        <v>79987</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
@@ -2112,48 +2112,48 @@
         <v>47252</v>
       </c>
       <c r="I44" t="n">
-        <v>62.52</v>
+        <v>111.1</v>
       </c>
       <c r="J44" t="n">
-        <v>62.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>142124</v>
+        <v>102636</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>4Q6489</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>31305</v>
+        <v>53333</v>
       </c>
       <c r="I45" t="n">
-        <v>185.14</v>
+        <v>11.39</v>
       </c>
       <c r="J45" t="n">
-        <v>185.13</v>
+        <v>11.39</v>
       </c>
     </row>
     <row r="46">
@@ -2171,11 +2171,11 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>147194</v>
+        <v>110370</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
@@ -2185,51 +2185,51 @@
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>33928</v>
+        <v>47252</v>
       </c>
       <c r="I46" t="n">
-        <v>7.99</v>
+        <v>62.52</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>148828</v>
+        <v>142124</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G47" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>792019</v>
+        <v>31305</v>
       </c>
       <c r="I47" t="n">
-        <v>93.70999999999999</v>
+        <v>185.14</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="48">
@@ -2239,32 +2239,32 @@
         </is>
       </c>
       <c r="B48" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>153194</v>
+        <v>147194</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0000293059</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G48" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>789423</v>
+        <v>33928</v>
       </c>
       <c r="I48" t="n">
-        <v>64.01000000000001</v>
+        <v>7.99</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2273,23 +2273,23 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>155970</v>
+        <v>148828</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -2299,13 +2299,13 @@
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>789423</v>
+        <v>792019</v>
       </c>
       <c r="I49" t="n">
-        <v>283.62</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J49" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -2315,111 +2315,111 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>81973</v>
+        <v>153194</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>0000293059</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G50" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H50" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I50" t="n">
-        <v>6.24</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="J50" t="n">
-        <v>6.24</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>106</v>
+        <v>39</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>102393</v>
+        <v>155970</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>4O3174</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
-        <v>46357</v>
+        <v>46508</v>
       </c>
       <c r="G51" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H51" t="n">
-        <v>53333</v>
+        <v>789423</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
+        <v>283.62</v>
       </c>
       <c r="J51" t="n">
-        <v>2.02</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>142672</v>
+        <v>81973</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I52" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
       <c r="J52" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="53">
@@ -2429,57 +2429,57 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>142886</v>
+        <v>102393</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H53" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I53" t="n">
-        <v>65.25</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>32.63</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>153194</v>
+        <v>142672</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
@@ -2489,35 +2489,35 @@
         <v>46259</v>
       </c>
       <c r="H54" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I54" t="n">
-        <v>155.28</v>
+        <v>39.31</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>155919</v>
+        <v>142886</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
@@ -2530,86 +2530,86 @@
         <v>789423</v>
       </c>
       <c r="I55" t="n">
-        <v>158.77</v>
+        <v>65.25</v>
       </c>
       <c r="J55" t="n">
-        <v>158.77</v>
+        <v>32.63</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>159083</v>
+        <v>153194</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G56" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H56" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I56" t="n">
-        <v>0</v>
+        <v>155.28</v>
       </c>
       <c r="J56" t="n">
-        <v>88.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>120</v>
+        <v>39</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>17310</v>
+        <v>155919</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>B25E1014</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G57" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H57" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I57" t="n">
-        <v>49.4</v>
+        <v>158.77</v>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="58">
@@ -2619,35 +2619,35 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>55476</v>
+        <v>159083</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H58" t="n">
-        <v>30791</v>
+        <v>794365</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>85.26000000000001</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="59">
@@ -2657,35 +2657,35 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>58</v>
+        <v>120</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>66958</v>
+        <v>17310</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>B25E1014</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H59" t="n">
-        <v>789525</v>
+        <v>47252</v>
       </c>
       <c r="I59" t="n">
-        <v>59.39</v>
+        <v>49.4</v>
       </c>
       <c r="J59" t="n">
-        <v>59.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
@@ -2695,35 +2695,35 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>92720</v>
+        <v>55476</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H60" t="n">
-        <v>37273</v>
+        <v>30791</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>6.88</v>
+        <v>85.26000000000001</v>
       </c>
     </row>
     <row r="61">
@@ -2733,175 +2733,175 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>100471</v>
+        <v>66958</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>4P2788</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H61" t="n">
-        <v>53333</v>
+        <v>789525</v>
       </c>
       <c r="I61" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
       <c r="J61" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>113662</v>
+        <v>92720</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>OB1115</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H62" t="n">
-        <v>31267</v>
+        <v>37273</v>
       </c>
       <c r="I62" t="n">
-        <v>100.89</v>
+        <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>37.31</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>140760</v>
+        <v>100471</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H63" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I63" t="n">
-        <v>37.39</v>
+        <v>126.28</v>
       </c>
       <c r="J63" t="n">
-        <v>37.39</v>
+        <v>126.28</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>125</v>
+        <v>38</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>145507</v>
+        <v>113662</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>OB1115</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>46485</v>
+        <v>46478</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H64" t="n">
-        <v>47252</v>
+        <v>31267</v>
       </c>
       <c r="I64" t="n">
-        <v>0</v>
+        <v>100.89</v>
       </c>
       <c r="J64" t="n">
-        <v>26.34</v>
+        <v>37.31</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>142</v>
+        <v>111</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>145709</v>
+        <v>140760</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>0000277236</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G65" s="2" t="n">
         <v>46259</v>
@@ -2910,83 +2910,83 @@
         <v>789423</v>
       </c>
       <c r="I65" t="n">
-        <v>49.42</v>
+        <v>37.39</v>
       </c>
       <c r="J65" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>38</v>
+        <v>125</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>150514</v>
+        <v>145507</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>4T3212</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>46508</v>
+        <v>46485</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H66" t="n">
-        <v>53333</v>
+        <v>47252</v>
       </c>
       <c r="I66" t="n">
-        <v>132.25</v>
+        <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>132.25</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>157673</v>
+        <v>145709</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>0525</t>
+          <t>0000277236</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H67" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I67" t="n">
-        <v>13.09</v>
+        <v>49.42</v>
       </c>
       <c r="J67" t="n">
         <v>0</v>
@@ -2995,77 +2995,77 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>160073</v>
+        <v>150514</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>4T3212</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H68" t="n">
-        <v>795751</v>
+        <v>53333</v>
       </c>
       <c r="I68" t="n">
-        <v>74.92</v>
+        <v>132.25</v>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>132.25</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>44733</v>
+        <v>157673</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>0525</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>46113</v>
+        <v>46419</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H69" t="n">
-        <v>790283</v>
+        <v>47252</v>
       </c>
       <c r="I69" t="n">
-        <v>27.55</v>
+        <v>13.09</v>
       </c>
       <c r="J69" t="n">
-        <v>27.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70">
@@ -3083,141 +3083,141 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>49964</v>
+        <v>160073</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G70" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H70" t="n">
-        <v>789228</v>
+        <v>795751</v>
       </c>
       <c r="I70" t="n">
-        <v>82.84999999999999</v>
+        <v>74.92</v>
       </c>
       <c r="J70" t="n">
-        <v>82.84999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>55204</v>
+        <v>44733</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>46447</v>
+        <v>46113</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H71" t="n">
-        <v>30791</v>
+        <v>790283</v>
       </c>
       <c r="I71" t="n">
-        <v>43.92</v>
+        <v>27.55</v>
       </c>
       <c r="J71" t="n">
-        <v>43.92</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>84824</v>
+        <v>49964</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H72" t="n">
-        <v>789662</v>
+        <v>789228</v>
       </c>
       <c r="I72" t="n">
-        <v>27.31</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J72" t="n">
-        <v>0</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>88358</v>
+        <v>55204</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H73" t="n">
-        <v>793056</v>
+        <v>30791</v>
       </c>
       <c r="I73" t="n">
-        <v>0</v>
+        <v>43.92</v>
       </c>
       <c r="J73" t="n">
-        <v>42.8</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="74">
@@ -3235,11 +3235,11 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>101583</v>
+        <v>84824</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>4V6234</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
@@ -3249,10 +3249,10 @@
         <v>46259</v>
       </c>
       <c r="H74" t="n">
-        <v>53333</v>
+        <v>789662</v>
       </c>
       <c r="I74" t="n">
-        <v>125.05</v>
+        <v>27.31</v>
       </c>
       <c r="J74" t="n">
         <v>0</v>
@@ -3261,175 +3261,175 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>105546</v>
+        <v>88358</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H75" t="n">
-        <v>789423</v>
+        <v>793056</v>
       </c>
       <c r="I75" t="n">
-        <v>186.49</v>
+        <v>0</v>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>106348</v>
+        <v>101583</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>4V6234</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H76" t="n">
-        <v>65455</v>
+        <v>53333</v>
       </c>
       <c r="I76" t="n">
-        <v>0</v>
+        <v>125.05</v>
       </c>
       <c r="J76" t="n">
-        <v>11.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>106364</v>
+        <v>105546</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H77" t="n">
-        <v>65455</v>
+        <v>789423</v>
       </c>
       <c r="I77" t="n">
-        <v>51.35</v>
+        <v>186.49</v>
       </c>
       <c r="J77" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>96</v>
+        <v>39</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>142645</v>
+        <v>106348</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H78" t="n">
-        <v>789429</v>
+        <v>65455</v>
       </c>
       <c r="I78" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
       <c r="J78" t="n">
-        <v>81.64</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>146095</v>
+        <v>106364</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
@@ -3439,51 +3439,51 @@
         <v>46259</v>
       </c>
       <c r="H79" t="n">
-        <v>790283</v>
+        <v>65455</v>
       </c>
       <c r="I79" t="n">
-        <v>8.15</v>
+        <v>51.35</v>
       </c>
       <c r="J79" t="n">
-        <v>20.67</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>147</v>
+        <v>96</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>148816</v>
+        <v>142645</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>25E17F</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G80" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H80" t="n">
-        <v>33928</v>
+        <v>789429</v>
       </c>
       <c r="I80" t="n">
-        <v>10.43</v>
+        <v>81.64</v>
       </c>
       <c r="J80" t="n">
-        <v>10.43</v>
+        <v>81.64</v>
       </c>
     </row>
     <row r="81">
@@ -3501,64 +3501,140 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>148823</v>
+        <v>146095</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>252535</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G81" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H81" t="n">
-        <v>33928</v>
+        <v>790283</v>
       </c>
       <c r="I81" t="n">
-        <v>53.82</v>
+        <v>8.15</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>147</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G82" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H82" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I82" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J82" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
           <t>PI</t>
         </is>
       </c>
-      <c r="B82" t="n">
+      <c r="B83" t="n">
         <v>39</v>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
-      <c r="D82" t="n">
+      <c r="D83" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G83" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H83" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I83" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>39</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
         <v>157761</v>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F82" s="2" t="n">
+      <c r="F84" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G82" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H82" t="n">
+      <c r="G84" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H84" t="n">
         <v>790808</v>
       </c>
-      <c r="I82" t="n">
-        <v>0</v>
-      </c>
-      <c r="J82" t="n">
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 17:30:04
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2881,23 +2881,23 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>111</v>
+        <v>38</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>140760</v>
+        <v>117650</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>4U6008</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
@@ -2907,13 +2907,13 @@
         <v>46259</v>
       </c>
       <c r="H65" t="n">
-        <v>789423</v>
+        <v>790808</v>
       </c>
       <c r="I65" t="n">
-        <v>37.39</v>
+        <v>27.71</v>
       </c>
       <c r="J65" t="n">
-        <v>37.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66">
@@ -2923,95 +2923,95 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>145507</v>
+        <v>140760</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>46485</v>
+        <v>46447</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H66" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I66" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
       <c r="J66" t="n">
-        <v>26.34</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>142</v>
+        <v>125</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>145709</v>
+        <v>145507</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>0000277236</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>46508</v>
+        <v>46485</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H67" t="n">
-        <v>789423</v>
+        <v>47252</v>
       </c>
       <c r="I67" t="n">
-        <v>49.42</v>
+        <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>0</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>38</v>
+        <v>142</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>150514</v>
+        <v>145709</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>4T3212</t>
+          <t>0000277236</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
@@ -3021,86 +3021,86 @@
         <v>46259</v>
       </c>
       <c r="H68" t="n">
-        <v>53333</v>
+        <v>789423</v>
       </c>
       <c r="I68" t="n">
-        <v>132.25</v>
+        <v>49.42</v>
       </c>
       <c r="J68" t="n">
-        <v>132.25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>125</v>
+        <v>38</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>157673</v>
+        <v>150514</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>0525</t>
+          <t>4T3212</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H69" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I69" t="n">
-        <v>13.09</v>
+        <v>132.25</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>132.25</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>160073</v>
+        <v>157673</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>0525</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G70" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H70" t="n">
-        <v>795751</v>
+        <v>47252</v>
       </c>
       <c r="I70" t="n">
-        <v>74.92</v>
+        <v>13.09</v>
       </c>
       <c r="J70" t="n">
         <v>0</v>
@@ -3109,77 +3109,77 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>120</v>
+        <v>39</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>44733</v>
+        <v>160073</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>46113</v>
+        <v>46447</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H71" t="n">
-        <v>790283</v>
+        <v>795751</v>
       </c>
       <c r="I71" t="n">
-        <v>27.55</v>
+        <v>74.92</v>
       </c>
       <c r="J71" t="n">
-        <v>27.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>39</v>
+        <v>120</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>49964</v>
+        <v>44733</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>46419</v>
+        <v>46113</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H72" t="n">
-        <v>789228</v>
+        <v>790283</v>
       </c>
       <c r="I72" t="n">
-        <v>82.84999999999999</v>
+        <v>27.55</v>
       </c>
       <c r="J72" t="n">
-        <v>82.84999999999999</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="73">
@@ -3197,87 +3197,87 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>55204</v>
+        <v>49964</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H73" t="n">
-        <v>30791</v>
+        <v>789228</v>
       </c>
       <c r="I73" t="n">
-        <v>43.92</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J73" t="n">
-        <v>43.92</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>84824</v>
+        <v>55204</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G74" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H74" t="n">
-        <v>789662</v>
+        <v>30791</v>
       </c>
       <c r="I74" t="n">
-        <v>27.31</v>
+        <v>43.92</v>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>88358</v>
+        <v>84824</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
@@ -3287,35 +3287,35 @@
         <v>46259</v>
       </c>
       <c r="H75" t="n">
-        <v>793056</v>
+        <v>789662</v>
       </c>
       <c r="I75" t="n">
-        <v>0</v>
+        <v>27.31</v>
       </c>
       <c r="J75" t="n">
-        <v>42.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>147</v>
+        <v>125</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>101583</v>
+        <v>88358</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>4V6234</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
@@ -3325,48 +3325,48 @@
         <v>46259</v>
       </c>
       <c r="H76" t="n">
-        <v>53333</v>
+        <v>793056</v>
       </c>
       <c r="I76" t="n">
-        <v>125.05</v>
+        <v>0</v>
       </c>
       <c r="J76" t="n">
-        <v>0</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>53</v>
+        <v>147</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>105546</v>
+        <v>101583</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>4V6234</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H77" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I77" t="n">
-        <v>186.49</v>
+        <v>125.05</v>
       </c>
       <c r="J77" t="n">
         <v>0</v>
@@ -3375,65 +3375,65 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>106348</v>
+        <v>105546</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>46478</v>
+        <v>46419</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H78" t="n">
-        <v>65455</v>
+        <v>789423</v>
       </c>
       <c r="I78" t="n">
-        <v>0</v>
+        <v>186.49</v>
       </c>
       <c r="J78" t="n">
-        <v>11.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>125</v>
+        <v>39</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>106364</v>
+        <v>106348</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G79" s="2" t="n">
         <v>46259</v>
@@ -3442,32 +3442,32 @@
         <v>65455</v>
       </c>
       <c r="I79" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
       <c r="J79" t="n">
-        <v>51.35</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>96</v>
+        <v>125</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>142645</v>
+        <v>106364</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
@@ -3477,13 +3477,13 @@
         <v>46259</v>
       </c>
       <c r="H80" t="n">
-        <v>789429</v>
+        <v>65455</v>
       </c>
       <c r="I80" t="n">
-        <v>81.64</v>
+        <v>51.35</v>
       </c>
       <c r="J80" t="n">
-        <v>81.64</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="81">
@@ -3501,65 +3501,65 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>146095</v>
+        <v>123358</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>2500058</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G81" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H81" t="n">
-        <v>790283</v>
+        <v>33928</v>
       </c>
       <c r="I81" t="n">
-        <v>8.15</v>
+        <v>13.21</v>
       </c>
       <c r="J81" t="n">
-        <v>20.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>147</v>
+        <v>96</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SILAS SALVIANO PRATI</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>148816</v>
+        <v>142645</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>25E17F</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G82" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H82" t="n">
-        <v>33928</v>
+        <v>789429</v>
       </c>
       <c r="I82" t="n">
-        <v>10.43</v>
+        <v>81.64</v>
       </c>
       <c r="J82" t="n">
-        <v>10.43</v>
+        <v>81.64</v>
       </c>
     </row>
     <row r="83">
@@ -3577,64 +3577,140 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>148823</v>
+        <v>146095</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>252535</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G83" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H83" t="n">
-        <v>33928</v>
+        <v>790283</v>
       </c>
       <c r="I83" t="n">
-        <v>53.82</v>
+        <v>8.15</v>
       </c>
       <c r="J83" t="n">
-        <v>0</v>
+        <v>20.67</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>147</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G84" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H84" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I84" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J84" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
           <t>PI</t>
         </is>
       </c>
-      <c r="B84" t="n">
+      <c r="B85" t="n">
         <v>39</v>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
-      <c r="D84" t="n">
+      <c r="D85" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G85" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H85" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I85" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>39</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
         <v>157761</v>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F84" s="2" t="n">
+      <c r="F86" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G84" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H84" t="n">
+      <c r="G86" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H86" t="n">
         <v>790808</v>
       </c>
-      <c r="I84" t="n">
-        <v>0</v>
-      </c>
-      <c r="J84" t="n">
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): batch update intraday vendas - 17:45:04
</commit_message>
<xml_diff>
--- a/data/vadas_validade_9_meses.xlsx
+++ b/data/vadas_validade_9_meses.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J86"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1124,7 +1124,7 @@
         <v>30791</v>
       </c>
       <c r="I18" t="n">
-        <v>20.04</v>
+        <v>26.72</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
@@ -2011,11 +2011,11 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>120</v>
+        <v>38</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2023,11 +2023,11 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>1876167</t>
+          <t>1876217</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>45870</v>
+        <v>46357</v>
       </c>
       <c r="G42" s="2" t="n">
         <v>46259</v>
@@ -2036,184 +2036,184 @@
         <v>30791</v>
       </c>
       <c r="I42" t="n">
-        <v>59.5</v>
+        <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>59.5</v>
+        <v>59.47</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>66958</v>
+        <v>64130</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>1876167</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
-        <v>46478</v>
+        <v>45870</v>
       </c>
       <c r="G43" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H43" t="n">
-        <v>789525</v>
+        <v>30791</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
+        <v>59.5</v>
       </c>
       <c r="J43" t="n">
-        <v>32.14</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>79987</v>
+        <v>66958</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>B25B1713</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="G44" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H44" t="n">
-        <v>47252</v>
+        <v>789525</v>
       </c>
       <c r="I44" t="n">
-        <v>111.1</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>32.14</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>102636</v>
+        <v>79987</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>4Q6489</t>
+          <t>B25B1713</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G45" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H45" t="n">
-        <v>53333</v>
+        <v>47252</v>
       </c>
       <c r="I45" t="n">
-        <v>11.39</v>
+        <v>111.1</v>
       </c>
       <c r="J45" t="n">
-        <v>11.39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>147</v>
+        <v>38</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>110370</v>
+        <v>102636</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>B25A1125</t>
+          <t>4Q6489</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="G46" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H46" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I46" t="n">
-        <v>62.52</v>
+        <v>11.39</v>
       </c>
       <c r="J46" t="n">
-        <v>62.52</v>
+        <v>11.39</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>142124</v>
+        <v>110370</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>A40A00525</t>
+          <t>B25A1125</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -2223,35 +2223,35 @@
         <v>46259</v>
       </c>
       <c r="H47" t="n">
-        <v>31305</v>
+        <v>47252</v>
       </c>
       <c r="I47" t="n">
-        <v>185.14</v>
+        <v>62.52</v>
       </c>
       <c r="J47" t="n">
-        <v>185.13</v>
+        <v>62.52</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>147194</v>
+        <v>142124</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>B24G9303</t>
+          <t>A40A00525</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -2261,13 +2261,13 @@
         <v>46259</v>
       </c>
       <c r="H48" t="n">
-        <v>33928</v>
+        <v>31305</v>
       </c>
       <c r="I48" t="n">
-        <v>7.99</v>
+        <v>185.14</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>185.13</v>
       </c>
     </row>
     <row r="49">
@@ -2285,24 +2285,24 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>148828</v>
+        <v>147194</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>CG76M026</t>
+          <t>B24G9303</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G49" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H49" t="n">
-        <v>792019</v>
+        <v>33928</v>
       </c>
       <c r="I49" t="n">
-        <v>93.70999999999999</v>
+        <v>7.99</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
@@ -2315,19 +2315,19 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>153194</v>
+        <v>148828</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>0000293059</t>
+          <t>CG76M026</t>
         </is>
       </c>
       <c r="F50" s="2" t="n">
@@ -2337,10 +2337,10 @@
         <v>46259</v>
       </c>
       <c r="H50" t="n">
-        <v>789423</v>
+        <v>792019</v>
       </c>
       <c r="I50" t="n">
-        <v>64.01000000000001</v>
+        <v>93.70999999999999</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
@@ -2349,23 +2349,23 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>39</v>
+        <v>142</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>155970</v>
+        <v>153194</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>KB040441</t>
+          <t>0000293059</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
@@ -2378,124 +2378,124 @@
         <v>789423</v>
       </c>
       <c r="I51" t="n">
-        <v>283.62</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="J51" t="n">
-        <v>283.62</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>81973</v>
+        <v>155970</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>B25A0083</t>
+          <t>KB040441</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G52" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H52" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I52" t="n">
-        <v>6.24</v>
+        <v>283.62</v>
       </c>
       <c r="J52" t="n">
-        <v>6.24</v>
+        <v>283.62</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>106</v>
+        <v>147</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>102393</v>
+        <v>414045</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>4O3174</t>
+          <t>964681</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
-        <v>46357</v>
+        <v>46388</v>
       </c>
       <c r="G53" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H53" t="n">
-        <v>53333</v>
+        <v>33928</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
+        <v>20.83</v>
       </c>
       <c r="J53" t="n">
-        <v>2.02</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>142672</v>
+        <v>81973</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>25E02W</t>
+          <t>B25A0083</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G54" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H54" t="n">
-        <v>789429</v>
+        <v>47252</v>
       </c>
       <c r="I54" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
       <c r="J54" t="n">
-        <v>39.31</v>
+        <v>6.24</v>
       </c>
     </row>
     <row r="55">
@@ -2505,57 +2505,57 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>142886</v>
+        <v>102393</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>0000269338</t>
+          <t>4O3174</t>
         </is>
       </c>
       <c r="F55" s="2" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="G55" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H55" t="n">
-        <v>789423</v>
+        <v>53333</v>
       </c>
       <c r="I55" t="n">
-        <v>65.25</v>
+        <v>0</v>
       </c>
       <c r="J55" t="n">
-        <v>32.63</v>
+        <v>2.02</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>153194</v>
+        <v>142672</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>0000302385</t>
+          <t>25E02W</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
@@ -2565,35 +2565,35 @@
         <v>46259</v>
       </c>
       <c r="H56" t="n">
-        <v>789423</v>
+        <v>789429</v>
       </c>
       <c r="I56" t="n">
-        <v>155.28</v>
+        <v>39.31</v>
       </c>
       <c r="J56" t="n">
-        <v>0</v>
+        <v>39.31</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>155919</v>
+        <v>142886</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>KC040431</t>
+          <t>0000269338</t>
         </is>
       </c>
       <c r="F57" s="2" t="n">
@@ -2606,86 +2606,86 @@
         <v>789423</v>
       </c>
       <c r="I57" t="n">
-        <v>158.77</v>
+        <v>65.25</v>
       </c>
       <c r="J57" t="n">
-        <v>158.77</v>
+        <v>32.63</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>125</v>
+        <v>53</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>159083</v>
+        <v>153194</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2504659</t>
+          <t>0000302385</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G58" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H58" t="n">
-        <v>794365</v>
+        <v>789423</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
+        <v>155.28</v>
       </c>
       <c r="J58" t="n">
-        <v>88.59999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>120</v>
+        <v>39</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>17310</v>
+        <v>155919</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>B25E1014</t>
+          <t>KC040431</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
-        <v>46508</v>
+        <v>46388</v>
       </c>
       <c r="G59" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H59" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I59" t="n">
-        <v>49.4</v>
+        <v>158.77</v>
       </c>
       <c r="J59" t="n">
-        <v>0</v>
+        <v>158.77</v>
       </c>
     </row>
     <row r="60">
@@ -2695,35 +2695,35 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>JOSE MARIA FERNANDES FONTENELE</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>55476</v>
+        <v>159083</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>07643382</t>
+          <t>2504659</t>
         </is>
       </c>
       <c r="F60" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G60" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H60" t="n">
-        <v>30791</v>
+        <v>794365</v>
       </c>
       <c r="I60" t="n">
         <v>0</v>
       </c>
       <c r="J60" t="n">
-        <v>85.26000000000001</v>
+        <v>88.59999999999999</v>
       </c>
     </row>
     <row r="61">
@@ -2733,35 +2733,35 @@
         </is>
       </c>
       <c r="B61" t="n">
-        <v>58</v>
+        <v>120</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>WESLEY DE OLIVEIRA PAZ</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>66958</v>
+        <v>17310</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>2503322</t>
+          <t>B25E1014</t>
         </is>
       </c>
       <c r="F61" s="2" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="G61" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H61" t="n">
-        <v>789525</v>
+        <v>47252</v>
       </c>
       <c r="I61" t="n">
-        <v>59.39</v>
+        <v>49.45</v>
       </c>
       <c r="J61" t="n">
-        <v>59.39</v>
+        <v>49.45</v>
       </c>
     </row>
     <row r="62">
@@ -2771,35 +2771,35 @@
         </is>
       </c>
       <c r="B62" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>JOSE MARIA FERNANDES FONTENELE</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>92720</v>
+        <v>55476</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>4V3334</t>
+          <t>07643382</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G62" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H62" t="n">
-        <v>37273</v>
+        <v>30791</v>
       </c>
       <c r="I62" t="n">
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>6.88</v>
+        <v>85.26000000000001</v>
       </c>
     </row>
     <row r="63">
@@ -2809,95 +2809,95 @@
         </is>
       </c>
       <c r="B63" t="n">
-        <v>120</v>
+        <v>58</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>WESLEY DE OLIVEIRA PAZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>100471</v>
+        <v>66958</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>4P2788</t>
+          <t>2503322</t>
         </is>
       </c>
       <c r="F63" s="2" t="n">
-        <v>46419</v>
+        <v>46478</v>
       </c>
       <c r="G63" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H63" t="n">
-        <v>53333</v>
+        <v>789525</v>
       </c>
       <c r="I63" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
       <c r="J63" t="n">
-        <v>126.28</v>
+        <v>59.39</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>38</v>
+        <v>147</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>113662</v>
+        <v>79502</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>OB1115</t>
+          <t>B25C1094</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="G64" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H64" t="n">
-        <v>31267</v>
+        <v>47252</v>
       </c>
       <c r="I64" t="n">
-        <v>100.89</v>
+        <v>131.65</v>
       </c>
       <c r="J64" t="n">
-        <v>37.31</v>
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>38</v>
+        <v>145</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BERNARDO TEIXEIRA COSTA NETO</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>117650</v>
+        <v>85529</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>4U6008</t>
+          <t>FKP04526</t>
         </is>
       </c>
       <c r="F65" s="2" t="n">
@@ -2907,10 +2907,10 @@
         <v>46259</v>
       </c>
       <c r="H65" t="n">
-        <v>790808</v>
+        <v>789661</v>
       </c>
       <c r="I65" t="n">
-        <v>27.71</v>
+        <v>54.21</v>
       </c>
       <c r="J65" t="n">
         <v>0</v>
@@ -2923,111 +2923,111 @@
         </is>
       </c>
       <c r="B66" t="n">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>140760</v>
+        <v>92720</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>0000273697</t>
+          <t>4V3334</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G66" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H66" t="n">
-        <v>789423</v>
+        <v>37273</v>
       </c>
       <c r="I66" t="n">
-        <v>37.39</v>
+        <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>37.39</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>145507</v>
+        <v>100471</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Q24G0052</t>
+          <t>4P2788</t>
         </is>
       </c>
       <c r="F67" s="2" t="n">
-        <v>46485</v>
+        <v>46419</v>
       </c>
       <c r="G67" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H67" t="n">
-        <v>47252</v>
+        <v>53333</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
+        <v>126.28</v>
       </c>
       <c r="J67" t="n">
-        <v>26.34</v>
+        <v>126.28</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>142</v>
+        <v>38</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>145709</v>
+        <v>113662</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>0000277236</t>
+          <t>OB1115</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>46508</v>
+        <v>46478</v>
       </c>
       <c r="G68" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H68" t="n">
-        <v>789423</v>
+        <v>31267</v>
       </c>
       <c r="I68" t="n">
-        <v>49.42</v>
+        <v>100.96</v>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>100.95</v>
       </c>
     </row>
     <row r="69">
@@ -3045,27 +3045,27 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>150514</v>
+        <v>117650</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>4T3212</t>
+          <t>4U6008</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G69" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H69" t="n">
-        <v>53333</v>
+        <v>790808</v>
       </c>
       <c r="I69" t="n">
-        <v>132.25</v>
+        <v>27.71</v>
       </c>
       <c r="J69" t="n">
-        <v>132.25</v>
+        <v>27.71</v>
       </c>
     </row>
     <row r="70">
@@ -3075,222 +3075,222 @@
         </is>
       </c>
       <c r="B70" t="n">
-        <v>125</v>
+        <v>111</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t xml:space="preserve">SUPERVISÃO HERTZ CE </t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>157673</v>
+        <v>140760</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>0525</t>
+          <t>0000273697</t>
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G70" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H70" t="n">
-        <v>47252</v>
+        <v>789423</v>
       </c>
       <c r="I70" t="n">
-        <v>13.09</v>
+        <v>37.39</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>37.39</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>160073</v>
+        <v>145507</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>NC052</t>
+          <t>Q24G0052</t>
         </is>
       </c>
       <c r="F71" s="2" t="n">
-        <v>46447</v>
+        <v>46485</v>
       </c>
       <c r="G71" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H71" t="n">
-        <v>795751</v>
+        <v>47252</v>
       </c>
       <c r="I71" t="n">
-        <v>74.92</v>
+        <v>0</v>
       </c>
       <c r="J71" t="n">
-        <v>0</v>
+        <v>26.34</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
+          <t>SUPERVISÃO HERTZ PE (PATRICIA AZEVEDO)</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>44733</v>
+        <v>145709</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>241868</t>
+          <t>0000277236</t>
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>46113</v>
+        <v>46508</v>
       </c>
       <c r="G72" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H72" t="n">
-        <v>790283</v>
+        <v>789423</v>
       </c>
       <c r="I72" t="n">
-        <v>27.55</v>
+        <v>49.42</v>
       </c>
       <c r="J72" t="n">
-        <v>27.55</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>BERNARDO TEIXEIRA COSTA NETO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>49964</v>
+        <v>150514</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>PL0771</t>
+          <t>4T3212</t>
         </is>
       </c>
       <c r="F73" s="2" t="n">
-        <v>46419</v>
+        <v>46508</v>
       </c>
       <c r="G73" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H73" t="n">
-        <v>789228</v>
+        <v>53333</v>
       </c>
       <c r="I73" t="n">
-        <v>82.84999999999999</v>
+        <v>132.25</v>
       </c>
       <c r="J73" t="n">
-        <v>82.84999999999999</v>
+        <v>132.25</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>55204</v>
+        <v>157673</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>08681216</t>
+          <t>0525</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="G74" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H74" t="n">
-        <v>30791</v>
+        <v>47252</v>
       </c>
       <c r="I74" t="n">
-        <v>43.92</v>
+        <v>13.09</v>
       </c>
       <c r="J74" t="n">
-        <v>43.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>84824</v>
+        <v>160073</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FKP06475</t>
+          <t>NC052</t>
         </is>
       </c>
       <c r="F75" s="2" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="G75" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H75" t="n">
-        <v>789662</v>
+        <v>795751</v>
       </c>
       <c r="I75" t="n">
-        <v>27.31</v>
+        <v>74.92</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
@@ -3299,175 +3299,175 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>NUBIA EDUARDA DA CRUZ SOUZA</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>88358</v>
+        <v>44733</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>GRA01137</t>
+          <t>241868</t>
         </is>
       </c>
       <c r="F76" s="2" t="n">
-        <v>46508</v>
+        <v>46113</v>
       </c>
       <c r="G76" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H76" t="n">
-        <v>793056</v>
+        <v>790283</v>
       </c>
       <c r="I76" t="n">
-        <v>0</v>
+        <v>27.55</v>
       </c>
       <c r="J76" t="n">
-        <v>42.8</v>
+        <v>27.55</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>101583</v>
+        <v>49964</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>4V6234</t>
+          <t>PL0771</t>
         </is>
       </c>
       <c r="F77" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G77" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H77" t="n">
-        <v>53333</v>
+        <v>789228</v>
       </c>
       <c r="I77" t="n">
-        <v>125.05</v>
+        <v>82.84999999999999</v>
       </c>
       <c r="J77" t="n">
-        <v>0</v>
+        <v>82.84999999999999</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>GVBA OL HERTZ LAZARO DE SA</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>105546</v>
+        <v>55204</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>0000270940</t>
+          <t>08681216</t>
         </is>
       </c>
       <c r="F78" s="2" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="G78" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H78" t="n">
-        <v>789423</v>
+        <v>30791</v>
       </c>
       <c r="I78" t="n">
-        <v>186.49</v>
+        <v>43.92</v>
       </c>
       <c r="J78" t="n">
-        <v>0</v>
+        <v>43.92</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>39</v>
+        <v>145</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>106348</v>
+        <v>71404</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>BR181245</t>
+          <t>4N1861</t>
         </is>
       </c>
       <c r="F79" s="2" t="n">
-        <v>46478</v>
+        <v>46357</v>
       </c>
       <c r="G79" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H79" t="n">
-        <v>65455</v>
+        <v>37273</v>
       </c>
       <c r="I79" t="n">
-        <v>0</v>
+        <v>116.58</v>
       </c>
       <c r="J79" t="n">
-        <v>11.29</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>125</v>
+        <v>147</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>FERNANDO NOBRE MARTINS</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>106364</v>
+        <v>84824</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>BR183284</t>
+          <t>FKP06475</t>
         </is>
       </c>
       <c r="F80" s="2" t="n">
@@ -3477,73 +3477,73 @@
         <v>46259</v>
       </c>
       <c r="H80" t="n">
-        <v>65455</v>
+        <v>789662</v>
       </c>
       <c r="I80" t="n">
-        <v>51.35</v>
+        <v>27.31</v>
       </c>
       <c r="J80" t="n">
-        <v>51.35</v>
+        <v>0</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>123358</v>
+        <v>88358</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>2500058</t>
+          <t>GRA01137</t>
         </is>
       </c>
       <c r="F81" s="2" t="n">
-        <v>46388</v>
+        <v>46508</v>
       </c>
       <c r="G81" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H81" t="n">
-        <v>33928</v>
+        <v>793056</v>
       </c>
       <c r="I81" t="n">
-        <v>13.21</v>
+        <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>0</v>
+        <v>42.8</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>96</v>
+        <v>147</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>SILAS SALVIANO PRATI</t>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>142645</v>
+        <v>101583</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>25E17F</t>
+          <t>4V6234</t>
         </is>
       </c>
       <c r="F82" s="2" t="n">
@@ -3553,73 +3553,73 @@
         <v>46259</v>
       </c>
       <c r="H82" t="n">
-        <v>789429</v>
+        <v>53333</v>
       </c>
       <c r="I82" t="n">
-        <v>81.64</v>
+        <v>125.05</v>
       </c>
       <c r="J82" t="n">
-        <v>81.64</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>GVBA OL HERTZ LAZARO DE SA</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>146095</v>
+        <v>105546</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>252535</t>
+          <t>0000270940</t>
         </is>
       </c>
       <c r="F83" s="2" t="n">
-        <v>46508</v>
+        <v>46419</v>
       </c>
       <c r="G83" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H83" t="n">
-        <v>790283</v>
+        <v>789423</v>
       </c>
       <c r="I83" t="n">
-        <v>8.15</v>
+        <v>186.49</v>
       </c>
       <c r="J83" t="n">
-        <v>20.67</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>147</v>
+        <v>39</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>148816</v>
+        <v>106348</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>T16725</t>
+          <t>BR181245</t>
         </is>
       </c>
       <c r="F84" s="2" t="n">
@@ -3629,51 +3629,51 @@
         <v>46259</v>
       </c>
       <c r="H84" t="n">
-        <v>33928</v>
+        <v>65455</v>
       </c>
       <c r="I84" t="n">
-        <v>10.43</v>
+        <v>0</v>
       </c>
       <c r="J84" t="n">
-        <v>10.43</v>
+        <v>11.29</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>39</v>
+        <v>125</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+          <t>FERNANDO NOBRE MARTINS</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>148823</v>
+        <v>106364</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>T15925</t>
+          <t>BR183284</t>
         </is>
       </c>
       <c r="F85" s="2" t="n">
-        <v>46447</v>
+        <v>46508</v>
       </c>
       <c r="G85" s="2" t="n">
         <v>46259</v>
       </c>
       <c r="H85" t="n">
-        <v>33928</v>
+        <v>65455</v>
       </c>
       <c r="I85" t="n">
-        <v>53.82</v>
+        <v>51.35</v>
       </c>
       <c r="J85" t="n">
-        <v>0</v>
+        <v>51.35</v>
       </c>
     </row>
     <row r="86">
@@ -3691,26 +3691,216 @@
         </is>
       </c>
       <c r="D86" t="n">
+        <v>123358</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>2500058</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>46388</v>
+      </c>
+      <c r="G86" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H86" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I86" t="n">
+        <v>13.21</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>96</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>SILAS SALVIANO PRATI</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>142645</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>25E17F</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G87" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H87" t="n">
+        <v>789429</v>
+      </c>
+      <c r="I87" t="n">
+        <v>81.64</v>
+      </c>
+      <c r="J87" t="n">
+        <v>81.64</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>39</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>146095</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>252535</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>46508</v>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H88" t="n">
+        <v>790283</v>
+      </c>
+      <c r="I88" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="J88" t="n">
+        <v>20.67</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>147</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>ALEXSANDRO P DA VEIGA PACHECO (FARMA PE)</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>148816</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>T16725</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="n">
+        <v>46478</v>
+      </c>
+      <c r="G89" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H89" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I89" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="J89" t="n">
+        <v>10.43</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>39</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>148823</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>T15925</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>46447</v>
+      </c>
+      <c r="G90" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H90" t="n">
+        <v>33928</v>
+      </c>
+      <c r="I90" t="n">
+        <v>53.82</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>39</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>SAYONARA CORDEIRO DA COSTA HOLANDA</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
         <v>157761</v>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>4O4518</t>
         </is>
       </c>
-      <c r="F86" s="2" t="n">
+      <c r="F91" s="2" t="n">
         <v>46357</v>
       </c>
-      <c r="G86" s="2" t="n">
-        <v>46259</v>
-      </c>
-      <c r="H86" t="n">
+      <c r="G91" s="2" t="n">
+        <v>46259</v>
+      </c>
+      <c r="H91" t="n">
         <v>790808</v>
       </c>
-      <c r="I86" t="n">
-        <v>0</v>
-      </c>
-      <c r="J86" t="n">
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
         <v>104.85</v>
       </c>
     </row>

</xml_diff>